<commit_message>
FIX: morning briefing exit=2 — build_data.py 180s timeout left tickers.json stale
morning_briefing.py aborts (exit 2) when infra/prototype/tickers.json is >24h
old. Root cause: build_data.py (writes tickers.json at scan end) intermittently
exceeded the 180s subprocess timeout in swing_trade.py on cold caches — log shows
repeated "v2 build_data.py timed out after 180s; v2 dashboard is now stale". When
it timed out, tickers.json wasn't refreshed → went stale (41h over a weekend) →
6:30 briefing aborted. Warm runtime is 106s; raised timeout to 360s (3.4x) so cold
runs finish. Refreshed tickers.json manually. MORNING-BRIEF-STALE.

Residual (environmental, not code): the Mac must be awake/online at 6:30 PT or the
Slack post fails DNS — affects all morning alerts, not just the briefing.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-06-15.xlsx
+++ b/cache/open_items_2026-06-15.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N295"/>
+  <dimension ref="A1:N296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -12176,7 +12176,7 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>SIGNAL-ALERTS-1</t>
+          <t>MORNING-BRIEF-STALE</t>
         </is>
       </c>
       <c r="C210" s="10" t="inlineStr">
@@ -12191,17 +12191,17 @@
       </c>
       <c r="E210" s="6" t="inlineStr">
         <is>
-          <t>Daily WATCH-to-BUY flip + new Elite Pick alerts</t>
+          <t>Morning briefing exit=2 (stale tickers.json)</t>
         </is>
       </c>
       <c r="F210" s="5" t="inlineStr">
         <is>
-          <t>Owner wanted Slack alerts for (a) firm BUY-candidate from entry-watcher, (b) names flipping to BUY day-over-day, (c) new Elite Picks per mode</t>
+          <t>morning_briefing.py aborts (exit 2) when infra/prototype/tickers.json &gt;24h old. Root cause: build_data.py (writes tickers.json at scan end) intermittently exceeds the 180s subprocess timeout in swing_trade.py on cold caches -&gt; tickers.json not refreshed -&gt; stale -&gt; briefing aborts. Compounded by transient Slack DNS failures when the Mac is asleep at 6:30am</t>
         </is>
       </c>
       <c r="G210" s="5" t="inlineStr">
         <is>
-          <t>entry_watch.py: distinct shadow BUY-CANDIDATE message (#a). signal_alerts.py: day-over-day diff of per-mode BUY lists (buy_candidates/medium_term_picks/long_term_picks) + elite_picks vs data/signal_alert_snapshot.json; grouped digest; LIVE to owner Slack with composite-score caveat; launchd com.swingtrade.signal-alerts 7:15 PT daily. Zero EODHD</t>
+          <t>Raised build_data.py subprocess timeout 180-&gt;360s in swing_trade.py (2x headroom). Manually refreshed tickers.json. Residual: machine must be awake/online at 6:30 PT for briefing+all alerts to post</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr"/>
@@ -12219,7 +12219,7 @@
       </c>
       <c r="M210" s="3" t="inlineStr">
         <is>
-          <t>116e27f63</t>
+          <t>e7721f05c</t>
         </is>
       </c>
       <c r="N210" s="8" t="inlineStr"/>
@@ -12230,7 +12230,7 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>WEEKEND-PHANTOMS</t>
+          <t>SIGNAL-ALERTS-1</t>
         </is>
       </c>
       <c r="C211" s="10" t="inlineStr">
@@ -12240,22 +12240,22 @@
       </c>
       <c r="D211" s="5" t="inlineStr">
         <is>
-          <t>Audit Trail / Data Quality</t>
+          <t>Alerts</t>
         </is>
       </c>
       <c r="E211" s="6" t="inlineStr">
         <is>
-          <t>Weekend pick_dates (Sat/Sun) in audit ledger</t>
+          <t>Daily WATCH-to-BUY flip + new Elite Pick alerts</t>
         </is>
       </c>
       <c r="F211" s="5" t="inlineStr">
         <is>
-          <t>signal_log writes pick_date as today.isoformat() — when scan runs on weekend (manual rerun), produces Sat/Sun dates EODHD can't price. 355 such phantoms in ledger. Fix: snap weekend dates forward to next Monday at both write-time (signal_tracker.log_signals) and build-time (build_audit_ledger.py). Preserves original via pick_date_orig field</t>
+          <t>Owner wanted Slack alerts for (a) firm BUY-candidate from entry-watcher, (b) names flipping to BUY day-over-day, (c) new Elite Picks per mode</t>
         </is>
       </c>
       <c r="G211" s="5" t="inlineStr">
         <is>
-          <t>signal_tracker.py log_signals dow snap + build_audit_ledger.py _compute_returns_for_ticker snap-forward · 353 records normalized · 2 residual edge cases</t>
+          <t>entry_watch.py: distinct shadow BUY-CANDIDATE message (#a). signal_alerts.py: day-over-day diff of per-mode BUY lists (buy_candidates/medium_term_picks/long_term_picks) + elite_picks vs data/signal_alert_snapshot.json; grouped digest; LIVE to owner Slack with composite-score caveat; launchd com.swingtrade.signal-alerts 7:15 PT daily. Zero EODHD</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr"/>
@@ -12268,23 +12268,23 @@
       </c>
       <c r="L211" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr">
         <is>
-          <t>e48edac16</t>
+          <t>116e27f63</t>
         </is>
       </c>
       <c r="N211" s="8" t="inlineStr"/>
     </row>
-    <row r="212" ht="75" customHeight="1">
+    <row r="212" ht="90" customHeight="1">
       <c r="A212" s="2" t="n">
         <v>211</v>
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>BT-GUARD-1</t>
+          <t>WEEKEND-PHANTOMS</t>
         </is>
       </c>
       <c r="C212" s="10" t="inlineStr">
@@ -12294,22 +12294,22 @@
       </c>
       <c r="D212" s="5" t="inlineStr">
         <is>
-          <t>Backtest Infrastructure</t>
+          <t>Audit Trail / Data Quality</t>
         </is>
       </c>
       <c r="E212" s="6" t="inlineStr">
         <is>
-          <t>Backtest min_score guard rail</t>
+          <t>Weekend pick_dates (Sat/Sun) in audit ledger</t>
         </is>
       </c>
       <c r="F212" s="5" t="inlineStr">
         <is>
-          <t>Users (and Claude sessions) repeatedly ran 252d backtests with --min-score 65 (live threshold) producing 0 BUYs across all 252 days. Historical scoring is structurally suppressed because sentiment/options/catalyst pillars depend on real-time data not in EODHD backfill.</t>
+          <t>signal_log writes pick_date as today.isoformat() — when scan runs on weekend (manual rerun), produces Sat/Sun dates EODHD can't price. 355 such phantoms in ledger. Fix: snap weekend dates forward to next Monday at both write-time (signal_tracker.log_signals) and build-time (build_audit_ledger.py). Preserves original via pick_date_orig field</t>
         </is>
       </c>
       <c r="G212" s="5" t="inlineStr">
         <is>
-          <t>backtest.py main() now warns loudly when --min-score &gt; 55 (backtest-safe floor). New --accept-low-buys flag silences the warning for legitimate grid-search explorations. --smoke bypasses the guard. Plus diagnostic doc: docs/backtest_historical_scoring_diagnostic.md.</t>
+          <t>signal_tracker.py log_signals dow snap + build_audit_ledger.py _compute_returns_for_ticker snap-forward · 353 records normalized · 2 residual edge cases</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr"/>
@@ -12327,18 +12327,18 @@
       </c>
       <c r="M212" s="3" t="inlineStr">
         <is>
-          <t>d754830</t>
+          <t>e48edac16</t>
         </is>
       </c>
       <c r="N212" s="8" t="inlineStr"/>
     </row>
-    <row r="213" ht="60" customHeight="1">
+    <row r="213" ht="75" customHeight="1">
       <c r="A213" s="2" t="n">
         <v>212</v>
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>LENS-PLAN-PERMODE-TARGETS</t>
+          <t>BT-GUARD-1</t>
         </is>
       </c>
       <c r="C213" s="10" t="inlineStr">
@@ -12348,22 +12348,22 @@
       </c>
       <c r="D213" s="5" t="inlineStr">
         <is>
-          <t>BullVeda · Plan</t>
+          <t>Backtest Infrastructure</t>
         </is>
       </c>
       <c r="E213" s="6" t="inlineStr">
         <is>
-          <t>lens-plan synthesizes per-mode targets by scaling swing levels</t>
+          <t>Backtest min_score guard rail</t>
         </is>
       </c>
       <c r="F213" s="5" t="inlineStr">
         <is>
-          <t>modeAdjust() in lens-plan.jsx scales swing stop/t1/t2 by fixed multipliers (POSITION 0.96/1.10/1.18, INVEST 0.84/1.32/1.58) instead of binding canonical per-mode targets.</t>
+          <t>Users (and Claude sessions) repeatedly ran 252d backtests with --min-score 65 (live threshold) producing 0 BUYs across all 252 days. Historical scoring is structurally suppressed because sentiment/options/catalyst pillars depend on real-time data not in EODHD backfill.</t>
         </is>
       </c>
       <c r="G213" s="5" t="inlineStr">
         <is>
-          <t>Bind per-mode stop/T1/T2/RR from /api/trade_engine?mode= (already fetched by Overview into STATE.payloads). Verdict already fixed to bind decisionsByMode 2026-06-09.</t>
+          <t>backtest.py main() now warns loudly when --min-score &gt; 55 (backtest-safe floor). New --accept-low-buys flag silences the warning for legitimate grid-search explorations. --smoke bypasses the guard. Plus diagnostic doc: docs/backtest_historical_scoring_diagnostic.md.</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr"/>
@@ -12376,23 +12376,23 @@
       </c>
       <c r="L213" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M213" s="3" t="inlineStr">
         <is>
-          <t>99cff7117</t>
+          <t>d754830</t>
         </is>
       </c>
       <c r="N213" s="8" t="inlineStr"/>
     </row>
-    <row r="214" ht="45" customHeight="1">
+    <row r="214" ht="60" customHeight="1">
       <c r="A214" s="2" t="n">
         <v>213</v>
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>SURFACE-WATCHLIST-MOCK</t>
+          <t>LENS-PLAN-PERMODE-TARGETS</t>
         </is>
       </c>
       <c r="C214" s="10" t="inlineStr">
@@ -12402,22 +12402,22 @@
       </c>
       <c r="D214" s="5" t="inlineStr">
         <is>
-          <t>BullVeda · Watchlist</t>
+          <t>BullVeda · Plan</t>
         </is>
       </c>
       <c r="E214" s="6" t="inlineStr">
         <is>
-          <t>surface-watchlist enrichWL fabricates row data from charCodeAt</t>
+          <t>lens-plan synthesizes per-mode targets by scaling swing levels</t>
         </is>
       </c>
       <c r="F214" s="5" t="inlineStr">
         <is>
-          <t>enrichWL() synthesizes rs/rvol/rr/earn/iv/wlb/n/pf/insider/sent (and conviction tier) from sym char codes — mock, not real data.</t>
+          <t>modeAdjust() in lens-plan.jsx scales swing stop/t1/t2 by fixed multipliers (POSITION 0.96/1.10/1.18, INVEST 0.84/1.32/1.58) instead of binding canonical per-mode targets.</t>
         </is>
       </c>
       <c r="G214" s="5" t="inlineStr">
         <is>
-          <t>Wire enrichWL to the real universe row via BV.scanRow; bind conviction_tier instead of deriving from score.</t>
+          <t>Bind per-mode stop/T1/T2/RR from /api/trade_engine?mode= (already fetched by Overview into STATE.payloads). Verdict already fixed to bind decisionsByMode 2026-06-09.</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr"/>
@@ -12446,7 +12446,7 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-1</t>
+          <t>SURFACE-WATCHLIST-MOCK</t>
         </is>
       </c>
       <c r="C215" s="10" t="inlineStr">
@@ -12456,22 +12456,22 @@
       </c>
       <c r="D215" s="5" t="inlineStr">
         <is>
-          <t>Choice C Strategy</t>
+          <t>BullVeda · Watchlist</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
         <is>
-          <t>Design doc — docs/strategy_defensive_rotation.md</t>
+          <t>surface-watchlist enrichWL fabricates row data from charCodeAt</t>
         </is>
       </c>
       <c r="F215" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 of Defensive Rotation sleeve build</t>
+          <t>enrichWL() synthesizes rs/rvol/rr/earn/iv/wlb/n/pf/insider/sent (and conviction tier) from sym char codes — mock, not real data.</t>
         </is>
       </c>
       <c r="G215" s="5" t="inlineStr">
         <is>
-          <t>Full design: mechanism, triggers, universe, validation plan</t>
+          <t>Wire enrichWL to the real universe row via BV.scanRow; bind conviction_tier instead of deriving from score.</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr"/>
@@ -12484,12 +12484,12 @@
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M215" s="3" t="inlineStr">
         <is>
-          <t>399922797</t>
+          <t>99cff7117</t>
         </is>
       </c>
       <c r="N215" s="8" t="inlineStr"/>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-2</t>
+          <t>DEFROT-1</t>
         </is>
       </c>
       <c r="C216" s="10" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="E216" s="6" t="inlineStr">
         <is>
-          <t>Config block — defensive_rotation_sleeve</t>
+          <t>Design doc — docs/strategy_defensive_rotation.md</t>
         </is>
       </c>
       <c r="F216" s="5" t="inlineStr">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="G216" s="5" t="inlineStr">
         <is>
-          <t>Curated universe, regime gates, sizing, stops; default _enabled=false</t>
+          <t>Full design: mechanism, triggers, universe, validation plan</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr"/>
@@ -12554,7 +12554,7 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-3</t>
+          <t>DEFROT-2</t>
         </is>
       </c>
       <c r="C217" s="10" t="inlineStr">
@@ -12569,7 +12569,7 @@
       </c>
       <c r="E217" s="6" t="inlineStr">
         <is>
-          <t>Detector function — _detect_defensive_rotation</t>
+          <t>Config block — defensive_rotation_sleeve</t>
         </is>
       </c>
       <c r="F217" s="5" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="G217" s="5" t="inlineStr">
         <is>
-          <t>Universe + regime + SPY-50EMA + RS + beta + ATR gates with per-criterion audit</t>
+          <t>Curated universe, regime gates, sizing, stops; default _enabled=false</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr"/>
@@ -12608,7 +12608,7 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-4</t>
+          <t>DEFROT-3</t>
         </is>
       </c>
       <c r="C218" s="10" t="inlineStr">
@@ -12623,7 +12623,7 @@
       </c>
       <c r="E218" s="6" t="inlineStr">
         <is>
-          <t>Wire into analyze_ticker</t>
+          <t>Detector function — _detect_defensive_rotation</t>
         </is>
       </c>
       <c r="F218" s="5" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="G218" s="5" t="inlineStr">
         <is>
-          <t>Setup family override + trade plan override (1.0 ATR stop, T1+3, T2+6, hold 10-30d, regime exit on SPY 50EMA reclaim)</t>
+          <t>Universe + regime + SPY-50EMA + RS + beta + ATR gates with per-criterion audit</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr"/>
@@ -12662,7 +12662,7 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-5</t>
+          <t>DEFROT-4</t>
         </is>
       </c>
       <c r="C219" s="10" t="inlineStr">
@@ -12677,7 +12677,7 @@
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>Decision engine bypasses</t>
+          <t>Wire into analyze_ticker</t>
         </is>
       </c>
       <c r="F219" s="5" t="inlineStr">
@@ -12687,7 +12687,7 @@
       </c>
       <c r="G219" s="5" t="inlineStr">
         <is>
-          <t>regime_gate + entry_quality + fund_adequacy bypassed for Defensive Rotation family</t>
+          <t>Setup family override + trade plan override (1.0 ATR stop, T1+3, T2+6, hold 10-30d, regime exit on SPY 50EMA reclaim)</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr"/>
@@ -12716,7 +12716,7 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-6</t>
+          <t>DEFROT-5</t>
         </is>
       </c>
       <c r="C220" s="10" t="inlineStr">
@@ -12731,7 +12731,7 @@
       </c>
       <c r="E220" s="6" t="inlineStr">
         <is>
-          <t>Universe coverage</t>
+          <t>Decision engine bypasses</t>
         </is>
       </c>
       <c r="F220" s="5" t="inlineStr">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="G220" s="5" t="inlineStr">
         <is>
-          <t>XLP, TLT, IEF added to custom_watchlist (XLU/XLV/GLD already present)</t>
+          <t>regime_gate + entry_quality + fund_adequacy bypassed for Defensive Rotation family</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr"/>
@@ -12770,7 +12770,7 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-7</t>
+          <t>DEFROT-6</t>
         </is>
       </c>
       <c r="C221" s="10" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="E221" s="6" t="inlineStr">
         <is>
-          <t>Smoke test + commit</t>
+          <t>Universe coverage</t>
         </is>
       </c>
       <c r="F221" s="5" t="inlineStr">
@@ -12795,7 +12795,7 @@
       </c>
       <c r="G221" s="5" t="inlineStr">
         <is>
-          <t>All 4 detector tests pass; ready for Phase 1 paper validation</t>
+          <t>XLP, TLT, IEF added to custom_watchlist (XLU/XLV/GLD already present)</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr"/>
@@ -12824,7 +12824,7 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-1</t>
+          <t>DEFROT-7</t>
         </is>
       </c>
       <c r="C222" s="10" t="inlineStr">
@@ -12839,17 +12839,17 @@
       </c>
       <c r="E222" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion design doc</t>
+          <t>Smoke test + commit</t>
         </is>
       </c>
       <c r="F222" s="5" t="inlineStr">
         <is>
-          <t>Sleeve build</t>
+          <t>Phase 1 of Defensive Rotation sleeve build</t>
         </is>
       </c>
       <c r="G222" s="5" t="inlineStr">
         <is>
-          <t>docs/strategy_mean_reversion.md — full Jegadeesh 1990 mechanism + validation plan</t>
+          <t>All 4 detector tests pass; ready for Phase 1 paper validation</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr"/>
@@ -12867,7 +12867,7 @@
       </c>
       <c r="M222" s="3" t="inlineStr">
         <is>
-          <t>d0c6c4e04</t>
+          <t>399922797</t>
         </is>
       </c>
       <c r="N222" s="8" t="inlineStr"/>
@@ -12878,7 +12878,7 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-2</t>
+          <t>MEANREV-1</t>
         </is>
       </c>
       <c r="C223" s="10" t="inlineStr">
@@ -12893,7 +12893,7 @@
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion config</t>
+          <t>Mean Reversion design doc</t>
         </is>
       </c>
       <c r="F223" s="5" t="inlineStr">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="G223" s="5" t="inlineStr">
         <is>
-          <t>RSI&lt;30, EMA200 floor, 3-5d hold; default _enabled=true (fires in current choppy regime)</t>
+          <t>docs/strategy_mean_reversion.md — full Jegadeesh 1990 mechanism + validation plan</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr"/>
@@ -12932,7 +12932,7 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-3</t>
+          <t>MEANREV-2</t>
         </is>
       </c>
       <c r="C224" s="10" t="inlineStr">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="E224" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion detector</t>
+          <t>Mean Reversion config</t>
         </is>
       </c>
       <c r="F224" s="5" t="inlineStr">
@@ -12957,7 +12957,7 @@
       </c>
       <c r="G224" s="5" t="inlineStr">
         <is>
-          <t>_detect_mean_reversion — 8-gate audit (regime/score/RSI/EMA200/recent_low/RVOL/ADV/earnings)</t>
+          <t>RSI&lt;30, EMA200 floor, 3-5d hold; default _enabled=true (fires in current choppy regime)</t>
         </is>
       </c>
       <c r="H224" s="2" t="inlineStr"/>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-4</t>
+          <t>MEANREV-3</t>
         </is>
       </c>
       <c r="C225" s="10" t="inlineStr">
@@ -13001,7 +13001,7 @@
       </c>
       <c r="E225" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion wiring</t>
+          <t>Mean Reversion detector</t>
         </is>
       </c>
       <c r="F225" s="5" t="inlineStr">
@@ -13011,7 +13011,7 @@
       </c>
       <c r="G225" s="5" t="inlineStr">
         <is>
-          <t>Setup family override + plan (1.0 ATR stop, +3/+5% T1/T2, 3-5d hold, hard time-stop)</t>
+          <t>_detect_mean_reversion — 8-gate audit (regime/score/RSI/EMA200/recent_low/RVOL/ADV/earnings)</t>
         </is>
       </c>
       <c r="H225" s="2" t="inlineStr"/>
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-5</t>
+          <t>MEANREV-4</t>
         </is>
       </c>
       <c r="C226" s="10" t="inlineStr">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="E226" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion bypass</t>
+          <t>Mean Reversion wiring</t>
         </is>
       </c>
       <c r="F226" s="5" t="inlineStr">
@@ -13065,7 +13065,7 @@
       </c>
       <c r="G226" s="5" t="inlineStr">
         <is>
-          <t>entry_quality bypass (EXTENDED-down IS the trigger)</t>
+          <t>Setup family override + plan (1.0 ATR stop, +3/+5% T1/T2, 3-5d hold, hard time-stop)</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr"/>
@@ -13094,7 +13094,7 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-6</t>
+          <t>MEANREV-5</t>
         </is>
       </c>
       <c r="C227" s="10" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="E227" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion smoke test</t>
+          <t>Mean Reversion bypass</t>
         </is>
       </c>
       <c r="F227" s="5" t="inlineStr">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="G227" s="5" t="inlineStr">
         <is>
-          <t>4 detector tests pass — fired=True on choppy+RSI=25+EMA200, rejected on RSI=55/below-EMA200/trending</t>
+          <t>entry_quality bypass (EXTENDED-down IS the trigger)</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr"/>
@@ -13148,7 +13148,7 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>PEAD-1</t>
+          <t>MEANREV-6</t>
         </is>
       </c>
       <c r="C228" s="10" t="inlineStr">
@@ -13163,7 +13163,7 @@
       </c>
       <c r="E228" s="6" t="inlineStr">
         <is>
-          <t>PEAD design doc</t>
+          <t>Mean Reversion smoke test</t>
         </is>
       </c>
       <c r="F228" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="G228" s="5" t="inlineStr">
         <is>
-          <t>docs/strategy_pead.md — Bernard-Thomas 1989, all-regime catalyst sleeve</t>
+          <t>4 detector tests pass — fired=True on choppy+RSI=25+EMA200, rejected on RSI=55/below-EMA200/trending</t>
         </is>
       </c>
       <c r="H228" s="2" t="inlineStr"/>
@@ -13202,7 +13202,7 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>PEAD-2</t>
+          <t>PEAD-1</t>
         </is>
       </c>
       <c r="C229" s="10" t="inlineStr">
@@ -13217,7 +13217,7 @@
       </c>
       <c r="E229" s="6" t="inlineStr">
         <is>
-          <t>PEAD config</t>
+          <t>PEAD design doc</t>
         </is>
       </c>
       <c r="F229" s="5" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="G229" s="5" t="inlineStr">
         <is>
-          <t>Day1-3 post-earnings, EPS+5/Rev+2/Gap+3/Revisions&gt;=2, full Kelly with regime caps</t>
+          <t>docs/strategy_pead.md — Bernard-Thomas 1989, all-regime catalyst sleeve</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr"/>
@@ -13256,7 +13256,7 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>PEAD-3</t>
+          <t>PEAD-2</t>
         </is>
       </c>
       <c r="C230" s="10" t="inlineStr">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="E230" s="6" t="inlineStr">
         <is>
-          <t>PEAD detector</t>
+          <t>PEAD config</t>
         </is>
       </c>
       <c r="F230" s="5" t="inlineStr">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="G230" s="5" t="inlineStr">
         <is>
-          <t>_detect_pead — 7-gate audit; regime-independent</t>
+          <t>Day1-3 post-earnings, EPS+5/Rev+2/Gap+3/Revisions&gt;=2, full Kelly with regime caps</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr"/>
@@ -13310,7 +13310,7 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>PEAD-4</t>
+          <t>PEAD-3</t>
         </is>
       </c>
       <c r="C231" s="10" t="inlineStr">
@@ -13325,7 +13325,7 @@
       </c>
       <c r="E231" s="6" t="inlineStr">
         <is>
-          <t>PEAD wiring</t>
+          <t>PEAD detector</t>
         </is>
       </c>
       <c r="F231" s="5" t="inlineStr">
@@ -13335,7 +13335,7 @@
       </c>
       <c r="G231" s="5" t="inlineStr">
         <is>
-          <t>Setup family override + plan (1.0 ATR stop, +5/+10/+15 targets, 10-30d drift hold)</t>
+          <t>_detect_pead — 7-gate audit; regime-independent</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr"/>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>PEAD-5</t>
+          <t>PEAD-4</t>
         </is>
       </c>
       <c r="C232" s="10" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="E232" s="6" t="inlineStr">
         <is>
-          <t>PEAD bypasses</t>
+          <t>PEAD wiring</t>
         </is>
       </c>
       <c r="F232" s="5" t="inlineStr">
@@ -13389,7 +13389,7 @@
       </c>
       <c r="G232" s="5" t="inlineStr">
         <is>
-          <t>regime_gate bypassed (catalyst regime-independent), entry_quality bypassed (gap-up IS trigger)</t>
+          <t>Setup family override + plan (1.0 ATR stop, +5/+10/+15 targets, 10-30d drift hold)</t>
         </is>
       </c>
       <c r="H232" s="2" t="inlineStr"/>
@@ -13418,7 +13418,7 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>PEAD-6</t>
+          <t>PEAD-5</t>
         </is>
       </c>
       <c r="C233" s="10" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>PEAD smoke test</t>
+          <t>PEAD bypasses</t>
         </is>
       </c>
       <c r="F233" s="5" t="inlineStr">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G233" s="5" t="inlineStr">
         <is>
-          <t>Perfect-setup test fires with all 7 audit checks ✓</t>
+          <t>regime_gate bypassed (catalyst regime-independent), entry_quality bypassed (gap-up IS trigger)</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr"/>
@@ -13472,7 +13472,7 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>CLEANUP-HOT-SECTORS</t>
+          <t>PEAD-6</t>
         </is>
       </c>
       <c r="C234" s="10" t="inlineStr">
@@ -13482,22 +13482,22 @@
       </c>
       <c r="D234" s="5" t="inlineStr">
         <is>
-          <t>Code Hygiene / Signal Scanner</t>
+          <t>Choice C Strategy</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
         <is>
-          <t>Remove dead panelHotSectors function</t>
+          <t>PEAD smoke test</t>
         </is>
       </c>
       <c r="F234" s="5" t="inlineStr">
         <is>
-          <t>User asked to remove Hot Sectors panel from grid earlier; function left in file as dead code. Removed 53 lines.</t>
+          <t>Sleeve build</t>
         </is>
       </c>
       <c r="G234" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner module · panelHotSectors() deleted</t>
+          <t>Perfect-setup test fires with all 7 audit checks ✓</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr"/>
@@ -13510,23 +13510,23 @@
       </c>
       <c r="L234" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="M234" s="3" t="inlineStr">
         <is>
-          <t>e48edac16</t>
+          <t>d0c6c4e04</t>
         </is>
       </c>
       <c r="N234" s="8" t="inlineStr"/>
     </row>
-    <row r="235" ht="105" customHeight="1">
+    <row r="235" ht="45" customHeight="1">
       <c r="A235" s="2" t="n">
         <v>234</v>
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>UI-CRYPTO-1</t>
+          <t>CLEANUP-HOT-SECTORS</t>
         </is>
       </c>
       <c r="C235" s="10" t="inlineStr">
@@ -13536,22 +13536,22 @@
       </c>
       <c r="D235" s="5" t="inlineStr">
         <is>
-          <t>Crypto Tab</t>
+          <t>Code Hygiene / Signal Scanner</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
         <is>
-          <t>20yr HF analyst Crypto tab rebuild</t>
+          <t>Remove dead panelHotSectors function</t>
         </is>
       </c>
       <c r="F235" s="5" t="inlineStr">
         <is>
-          <t>Crypto tab was stub with 4 cards of placeholder data. Needed a senior HF/Graham-Buffett/swing-trader fused lens for the 24/7 risk-asset bellwether.</t>
+          <t>User asked to remove Hot Sectors panel from grid earlier; function left in file as dead code. Removed 53 lines.</t>
         </is>
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>13-section renderCrypto in kairos.html: cycle posture banner (Pi-Cycle/MVRV-Z/NUPL/200wk MA), spot KPIs, Graham margin-of-safety floors (realized price, thermo-cap, cost of production, LTH/STH cost), ETH owner-earnings DCF, BTC hard-money compounding, stablecoin liquidity, macro drivers, spot ETF flows, derivatives tape, on-chain valuation composite, catalyst calendar, adjacent equities, L1/L2 rotation, regime-conditional playbook, pre-mortem.</t>
+          <t>kairos.html QuantScanner module · panelHotSectors() deleted</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr"/>
@@ -13569,18 +13569,18 @@
       </c>
       <c r="M235" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
+          <t>e48edac16</t>
         </is>
       </c>
       <c r="N235" s="8" t="inlineStr"/>
     </row>
-    <row r="236" ht="75" customHeight="1">
+    <row r="236" ht="105" customHeight="1">
       <c r="A236" s="2" t="n">
         <v>235</v>
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-T1CAT-1</t>
+          <t>UI-CRYPTO-1</t>
         </is>
       </c>
       <c r="C236" s="10" t="inlineStr">
@@ -13590,22 +13590,22 @@
       </c>
       <c r="D236" s="5" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Crypto Tab</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
         <is>
-          <t>T1 CATALYST pill read wrong field</t>
+          <t>20yr HF analyst Crypto tab rebuild</t>
         </is>
       </c>
       <c r="F236" s="5" t="inlineStr">
         <is>
-          <t>The scanner '⚡ T1 CATALYST' pill filtered t.tier===T1 (conviction_tier), not the catalyst tier. conviction_tier has 0 T1s on a no-BUY day (CPI blackout: AVOID 928/WATCH 133/T3 14), so the pill matched nothing — while catalyst_tier T1 = 239 names.</t>
+          <t>Crypto tab was stub with 4 cards of placeholder data. Needed a senior HF/Graham-Buffett/swing-trader fused lens for the 24/7 risk-asset bellwether.</t>
         </is>
       </c>
       <c r="G236" s="5" t="inlineStr">
         <is>
-          <t>Changed the pill filter to t.cat===T1 (catalyst tier, matching the displayed CAT column). Rebuilt.</t>
+          <t>13-section renderCrypto in kairos.html: cycle posture banner (Pi-Cycle/MVRV-Z/NUPL/200wk MA), spot KPIs, Graham margin-of-safety floors (realized price, thermo-cap, cost of production, LTH/STH cost), ETH owner-earnings DCF, BTC hard-money compounding, stablecoin liquidity, macro drivers, spot ETF flows, derivatives tape, on-chain valuation composite, catalyst calendar, adjacent equities, L1/L2 rotation, regime-conditional playbook, pre-mortem.</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr"/>
@@ -13618,12 +13618,12 @@
       </c>
       <c r="L236" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M236" s="3" t="inlineStr">
         <is>
-          <t>1d6fdb14a</t>
+          <t>696731a4d</t>
         </is>
       </c>
       <c r="N236" s="8" t="inlineStr"/>
@@ -13634,7 +13634,7 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>EODHD-EDGAR-FUNDAMENTALS</t>
+          <t>SCANNER-T1CAT-1</t>
         </is>
       </c>
       <c r="C237" s="10" t="inlineStr">
@@ -13644,22 +13644,22 @@
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
-          <t>Data / SEC EDGAR (future quality)</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
         <is>
-          <t>Offload fundamentals to SEC EDGAR (FIX 4)</t>
+          <t>T1 CATALYST pill read wrong field</t>
         </is>
       </c>
       <c r="F237" s="5" t="inlineStr">
         <is>
-          <t>new edgar_client.py behind data_fetcher interface; data.sec.gov companyfacts (User-Agent + &lt;=10 req/s); map XBRL tags to fundamentals.db; nightly batch. Quality upgrade (point-in-time, fixes audit #1/#4) + zeroes per-ticker EODHD fundamentals calls.</t>
+          <t>The scanner '⚡ T1 CATALYST' pill filtered t.tier===T1 (conviction_tier), not the catalyst tier. conviction_tier has 0 T1s on a no-BUY day (CPI blackout: AVOID 928/WATCH 133/T3 14), so the pill matched nothing — while catalyst_tier T1 = 239 names.</t>
         </is>
       </c>
       <c r="G237" s="5" t="inlineStr">
         <is>
-          <t>edgar_client.py + nightly batch</t>
+          <t>Changed the pill filter to t.cat===T1 (catalyst tier, matching the displayed CAT column). Rebuilt.</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr"/>
@@ -13672,12 +13672,12 @@
       </c>
       <c r="L237" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="M237" s="3" t="inlineStr">
         <is>
-          <t>5d05268ef</t>
+          <t>1d6fdb14a</t>
         </is>
       </c>
       <c r="N237" s="8" t="inlineStr"/>
@@ -13688,7 +13688,7 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-QUAL-REASON-1</t>
+          <t>EODHD-EDGAR-FUNDAMENTALS</t>
         </is>
       </c>
       <c r="C238" s="10" t="inlineStr">
@@ -13698,22 +13698,22 @@
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine</t>
+          <t>Data / SEC EDGAR (future quality)</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
         <is>
-          <t>Misleading entry_quality WATCH reason</t>
+          <t>Offload fundamentals to SEC EDGAR (FIX 4)</t>
         </is>
       </c>
       <c r="F238" s="5" t="inlineStr">
         <is>
-          <t>make_decision hardcoded 'broke through resistance, wait for next base' for ALL MISSED entries — false when stock is below recent high (BFH: MISSED via &gt;2 ATR over EMA21 but 2.1% BELOW 20d high)</t>
+          <t>new edgar_client.py behind data_fetcher interface; data.sec.gov companyfacts (User-Agent + &lt;=10 req/s); map XBRL tags to fundamentals.db; nightly batch. Quality upgrade (point-in-time, fixes audit #1/#4) + zeroes per-ticker EODHD fundamentals calls.</t>
         </is>
       </c>
       <c r="G238" s="5" t="inlineStr">
         <is>
-          <t>classify_entry_quality_detail() returns (label, live-distance reason) naming the actual trigger + honest 'still X% below resistance (not a breakout)' qualifier; threaded entry_quality_reason through make_decision + compute_decisions_by_mode</t>
+          <t>edgar_client.py + nightly batch</t>
         </is>
       </c>
       <c r="H238" s="2" t="inlineStr"/>
@@ -13726,23 +13726,23 @@
       </c>
       <c r="L238" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M238" s="3" t="inlineStr">
         <is>
-          <t>613f10e35</t>
+          <t>5d05268ef</t>
         </is>
       </c>
       <c r="N238" s="8" t="inlineStr"/>
     </row>
-    <row r="239" ht="60" customHeight="1">
+    <row r="239" ht="75" customHeight="1">
       <c r="A239" s="2" t="n">
         <v>238</v>
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>SETDETAIL-FALLBACK</t>
+          <t>ENTRY-QUAL-REASON-1</t>
         </is>
       </c>
       <c r="C239" s="10" t="inlineStr">
@@ -13752,22 +13752,22 @@
       </c>
       <c r="D239" s="5" t="inlineStr">
         <is>
-          <t>Detail UI / Routing</t>
+          <t>Decision Engine</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
         <is>
-          <t>setDetailTicker failed for R2000-only tickers</t>
+          <t>Misleading entry_quality WATCH reason</t>
         </is>
       </c>
       <c r="F239" s="5" t="inlineStr">
         <is>
-          <t>Clicking ML Edge picks not in scan bundle (HOOD, ARES, STEM etc.) printed '[kairos] ticker not in scan' and never opened. Now synthesizes minimal t row from window.__mlEdgeCache so detail page opens with _fromMlEdge:true flag</t>
+          <t>make_decision hardcoded 'broke through resistance, wait for next base' for ALL MISSED entries — false when stock is below recent high (BFH: MISSED via &gt;2 ATR over EMA21 but 2.1% BELOW 20d high)</t>
         </is>
       </c>
       <c r="G239" s="5" t="inlineStr">
         <is>
-          <t>kairos.html window.setDetailTicker fallback block</t>
+          <t>classify_entry_quality_detail() returns (label, live-distance reason) naming the actual trigger + honest 'still X% below resistance (not a breakout)' qualifier; threaded entry_quality_reason through make_decision + compute_decisions_by_mode</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr"/>
@@ -13780,12 +13780,12 @@
       </c>
       <c r="L239" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="M239" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
+          <t>613f10e35</t>
         </is>
       </c>
       <c r="N239" s="8" t="inlineStr"/>
@@ -13796,7 +13796,7 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>SETDETAIL-FALLBACK</t>
         </is>
       </c>
       <c r="C240" s="10" t="inlineStr">
@@ -13806,34 +13806,26 @@
       </c>
       <c r="D240" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Detail UI / Routing</t>
         </is>
       </c>
       <c r="E240" s="6" t="inlineStr">
         <is>
-          <t>Update CLAUDE.md with new tools</t>
+          <t>setDetailTicker failed for R2000-only tickers</t>
         </is>
       </c>
       <c r="F240" s="5" t="inlineStr">
         <is>
-          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
+          <t>Clicking ML Edge picks not in scan bundle (HOOD, ARES, STEM etc.) printed '[kairos] ticker not in scan' and never opened. Now synthesizes minimal t row from window.__mlEdgeCache so detail page opens with _fromMlEdge:true flag</t>
         </is>
       </c>
       <c r="G240" s="5" t="inlineStr">
         <is>
-          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
-        </is>
-      </c>
-      <c r="H240" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I240" s="5" t="inlineStr">
-        <is>
-          <t>Win: future Claude sessions discover new tools.</t>
-        </is>
-      </c>
+          <t>kairos.html window.setDetailTicker fallback block</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr"/>
+      <c r="I240" s="5" t="inlineStr"/>
       <c r="J240" s="5" t="inlineStr"/>
       <c r="K240" s="12" t="inlineStr">
         <is>
@@ -13842,27 +13834,23 @@
       </c>
       <c r="L240" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="M240" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N240" s="8" t="inlineStr">
-        <is>
-          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="241" ht="75" customHeight="1">
+          <t>27fd646b1</t>
+        </is>
+      </c>
+      <c r="N240" s="8" t="inlineStr"/>
+    </row>
+    <row r="241" ht="60" customHeight="1">
       <c r="A241" s="2" t="n">
         <v>240</v>
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C241" s="10" t="inlineStr">
@@ -13877,17 +13865,17 @@
       </c>
       <c r="E241" s="6" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
+          <t>Update CLAUDE.md with new tools</t>
         </is>
       </c>
       <c r="F241" s="5" t="inlineStr">
         <is>
-          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
+          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
         </is>
       </c>
       <c r="G241" s="5" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
+          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
         </is>
       </c>
       <c r="H241" s="2" t="inlineStr">
@@ -13897,14 +13885,10 @@
       </c>
       <c r="I241" s="5" t="inlineStr">
         <is>
-          <t>Win: clear activation procedure before flipping live.</t>
-        </is>
-      </c>
-      <c r="J241" s="5" t="inlineStr">
-        <is>
-          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
-        </is>
-      </c>
+          <t>Win: future Claude sessions discover new tools.</t>
+        </is>
+      </c>
+      <c r="J241" s="5" t="inlineStr"/>
       <c r="K241" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13917,12 +13901,12 @@
       </c>
       <c r="M241" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N241" s="8" t="inlineStr">
         <is>
-          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
         </is>
       </c>
     </row>
@@ -13932,7 +13916,7 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>TWO-LOG-DOC</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C242" s="10" t="inlineStr">
@@ -13947,22 +13931,34 @@
       </c>
       <c r="E242" s="6" t="inlineStr">
         <is>
-          <t>Two-log architecture (picks_history vs signal_log) was undocumented</t>
+          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
         </is>
       </c>
       <c r="F242" s="5" t="inlineStr">
         <is>
-          <t>Discovered 2026-05-10 during inflection diagnosis: cache/picks_history.json and data/signal_log.json track different realities (61.2% vs 12.7% recent WR). Tracker feedback reads picks_history; drift alerts read signal_log. Mis-attributing which log feeds which consumer wastes diagnostic time.</t>
+          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
         </is>
       </c>
       <c r="G242" s="5" t="inlineStr">
         <is>
-          <t>Add 'Two-Log Architecture' section to CLAUDE.md after EODHD section, with table mapping consumers + WR snapshots. Cross-reference portfolio_state.json as the ONLY real-trades log.</t>
-        </is>
-      </c>
-      <c r="H242" s="2" t="inlineStr"/>
-      <c r="I242" s="5" t="inlineStr"/>
-      <c r="J242" s="5" t="inlineStr"/>
+          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I242" s="5" t="inlineStr">
+        <is>
+          <t>Win: clear activation procedure before flipping live.</t>
+        </is>
+      </c>
+      <c r="J242" s="5" t="inlineStr">
+        <is>
+          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
+        </is>
+      </c>
       <c r="K242" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13970,23 +13966,27 @@
       </c>
       <c r="L242" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M242" s="3" t="inlineStr">
         <is>
-          <t>8b06e56ae</t>
-        </is>
-      </c>
-      <c r="N242" s="8" t="inlineStr"/>
-    </row>
-    <row r="243" ht="60" customHeight="1">
+          <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N242" s="8" t="inlineStr">
+        <is>
+          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="75" customHeight="1">
       <c r="A243" s="2" t="n">
         <v>242</v>
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>UI-HELP-1</t>
+          <t>TWO-LOG-DOC</t>
         </is>
       </c>
       <c r="C243" s="10" t="inlineStr">
@@ -13996,22 +13996,22 @@
       </c>
       <c r="D243" s="5" t="inlineStr">
         <is>
-          <t>Help System</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E243" s="6" t="inlineStr">
         <is>
-          <t>Help registry expanded 14 to 38 entries</t>
+          <t>Two-log architecture (picks_history vs signal_log) was undocumented</t>
         </is>
       </c>
       <c r="F243" s="5" t="inlineStr">
         <is>
-          <t>Help registry covered only workspace tabs. Detail sub-tabs and MarketsV2 ports had no help content.</t>
+          <t>Discovered 2026-05-10 during inflection diagnosis: cache/picks_history.json and data/signal_log.json track different realities (61.2% vs 12.7% recent WR). Tracker feedback reads picks_history; drift alerts read signal_log. Mis-attributing which log feeds which consumer wastes diagnostic time.</t>
         </is>
       </c>
       <c r="G243" s="5" t="inlineStr">
         <is>
-          <t>Added 24 new entries. kairosHelpFor threads isDetail through dispatcher — prefers detail_ namespace, falls back to bare key. Resolves portfolio workspace vs detail-subtab collision. MarketsV2 render block calls _injectHelpBtn.</t>
+          <t>Add 'Two-Log Architecture' section to CLAUDE.md after EODHD section, with table mapping consumers + WR snapshots. Cross-reference portfolio_state.json as the ONLY real-trades log.</t>
         </is>
       </c>
       <c r="H243" s="2" t="inlineStr"/>
@@ -14024,23 +14024,23 @@
       </c>
       <c r="L243" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
+          <t>8b06e56ae</t>
         </is>
       </c>
       <c r="N243" s="8" t="inlineStr"/>
     </row>
-    <row r="244" ht="45" customHeight="1">
+    <row r="244" ht="60" customHeight="1">
       <c r="A244" s="2" t="n">
         <v>243</v>
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>UI-HELP-1</t>
         </is>
       </c>
       <c r="C244" s="10" t="inlineStr">
@@ -14050,34 +14050,26 @@
       </c>
       <c r="D244" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Help System</t>
         </is>
       </c>
       <c r="E244" s="6" t="inlineStr">
         <is>
-          <t>Git committer.email set globally</t>
+          <t>Help registry expanded 14 to 38 entries</t>
         </is>
       </c>
       <c r="F244" s="5" t="inlineStr">
         <is>
-          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
+          <t>Help registry covered only workspace tabs. Detail sub-tabs and MarketsV2 ports had no help content.</t>
         </is>
       </c>
       <c r="G244" s="5" t="inlineStr">
         <is>
-          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
-        </is>
-      </c>
-      <c r="H244" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I244" s="5" t="inlineStr">
-        <is>
-          <t>Win: clean attribution in git log.</t>
-        </is>
-      </c>
+          <t>Added 24 new entries. kairosHelpFor threads isDetail through dispatcher — prefers detail_ namespace, falls back to bare key. Resolves portfolio workspace vs detail-subtab collision. MarketsV2 render block calls _injectHelpBtn.</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr"/>
+      <c r="I244" s="5" t="inlineStr"/>
       <c r="J244" s="5" t="inlineStr"/>
       <c r="K244" s="12" t="inlineStr">
         <is>
@@ -14086,27 +14078,23 @@
       </c>
       <c r="L244" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M244" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
-        </is>
-      </c>
-      <c r="N244" s="8" t="inlineStr">
-        <is>
-          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
-        </is>
-      </c>
-    </row>
-    <row r="245" ht="90" customHeight="1">
+          <t>696731a4d</t>
+        </is>
+      </c>
+      <c r="N244" s="8" t="inlineStr"/>
+    </row>
+    <row r="245" ht="45" customHeight="1">
       <c r="A245" s="2" t="n">
         <v>244</v>
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>UI-MLEDGE-1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="C245" s="10" t="inlineStr">
@@ -14116,26 +14104,34 @@
       </c>
       <c r="D245" s="5" t="inlineStr">
         <is>
-          <t>ML Edge Tab</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E245" s="6" t="inlineStr">
         <is>
-          <t>Theme switching + tf-* visual port</t>
+          <t>Git committer.email set globally</t>
         </is>
       </c>
       <c r="F245" s="5" t="inlineStr">
         <is>
-          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
+          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
         </is>
       </c>
       <c r="G245" s="5" t="inlineStr">
         <is>
-          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
-        </is>
-      </c>
-      <c r="H245" s="2" t="inlineStr"/>
-      <c r="I245" s="5" t="inlineStr"/>
+          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I245" s="5" t="inlineStr">
+        <is>
+          <t>Win: clean attribution in git log.</t>
+        </is>
+      </c>
       <c r="J245" s="5" t="inlineStr"/>
       <c r="K245" s="12" t="inlineStr">
         <is>
@@ -14144,23 +14140,27 @@
       </c>
       <c r="L245" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M245" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
-        </is>
-      </c>
-      <c r="N245" s="8" t="inlineStr"/>
-    </row>
-    <row r="246" ht="45" customHeight="1">
+          <t>4129e5565</t>
+        </is>
+      </c>
+      <c r="N245" s="8" t="inlineStr">
+        <is>
+          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="90" customHeight="1">
       <c r="A246" s="2" t="n">
         <v>245</v>
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>IPAD-2</t>
+          <t>UI-MLEDGE-1</t>
         </is>
       </c>
       <c r="C246" s="10" t="inlineStr">
@@ -14170,39 +14170,27 @@
       </c>
       <c r="D246" s="5" t="inlineStr">
         <is>
-          <t>Mobile / iPad</t>
+          <t>ML Edge Tab</t>
         </is>
       </c>
       <c r="E246" s="6" t="inlineStr">
         <is>
-          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
+          <t>Theme switching + tf-* visual port</t>
         </is>
       </c>
       <c r="F246" s="5" t="inlineStr">
         <is>
-          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
+          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
         </is>
       </c>
       <c r="G246" s="5" t="inlineStr">
         <is>
-          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
-        </is>
-      </c>
-      <c r="H246" s="2" t="inlineStr">
-        <is>
-          <t>15 min</t>
-        </is>
-      </c>
-      <c r="I246" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J246" s="5" t="inlineStr">
-        <is>
-          <t>Sub-task of IPAD-1.</t>
-        </is>
-      </c>
+          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr"/>
+      <c r="I246" s="5" t="inlineStr"/>
+      <c r="J246" s="5" t="inlineStr"/>
       <c r="K246" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14210,19 +14198,15 @@
       </c>
       <c r="L246" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr">
         <is>
-          <t>79fa01a75</t>
-        </is>
-      </c>
-      <c r="N246" s="8" t="inlineStr">
-        <is>
-          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
-        </is>
-      </c>
+          <t>696731a4d</t>
+        </is>
+      </c>
+      <c r="N246" s="8" t="inlineStr"/>
     </row>
     <row r="247" ht="45" customHeight="1">
       <c r="A247" s="2" t="n">
@@ -14230,7 +14214,7 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>SLACK-NEWSLETTER-MLALERT</t>
+          <t>IPAD-2</t>
         </is>
       </c>
       <c r="C247" s="10" t="inlineStr">
@@ -14240,27 +14224,39 @@
       </c>
       <c r="D247" s="5" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile / iPad</t>
         </is>
       </c>
       <c r="E247" s="6" t="inlineStr">
         <is>
-          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
+          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
         </is>
       </c>
       <c r="F247" s="5" t="inlineStr">
         <is>
-          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
+          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
         </is>
       </c>
       <c r="G247" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd + scripts/ml_alert_slack.py</t>
-        </is>
-      </c>
-      <c r="H247" s="2" t="inlineStr"/>
-      <c r="I247" s="5" t="inlineStr"/>
-      <c r="J247" s="5" t="inlineStr"/>
+          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="I247" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J247" s="5" t="inlineStr">
+        <is>
+          <t>Sub-task of IPAD-1.</t>
+        </is>
+      </c>
       <c r="K247" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14268,15 +14264,19 @@
       </c>
       <c r="L247" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr">
         <is>
-          <t>d1ea97913</t>
-        </is>
-      </c>
-      <c r="N247" s="8" t="inlineStr"/>
+          <t>79fa01a75</t>
+        </is>
+      </c>
+      <c r="N247" s="8" t="inlineStr">
+        <is>
+          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
+        </is>
+      </c>
     </row>
     <row r="248" ht="45" customHeight="1">
       <c r="A248" s="2" t="n">
@@ -14284,7 +14284,7 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>FORENSICS-WEEKLY-SLACK</t>
+          <t>SLACK-NEWSLETTER-MLALERT</t>
         </is>
       </c>
       <c r="C248" s="10" t="inlineStr">
@@ -14294,22 +14294,22 @@
       </c>
       <c r="D248" s="5" t="inlineStr">
         <is>
-          <t>Notifications / Audit</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E248" s="6" t="inlineStr">
         <is>
-          <t>Weekly pick-forensics Slack digest</t>
+          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
         </is>
       </c>
       <c r="F248" s="5" t="inlineStr">
         <is>
-          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
+          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
         </is>
       </c>
       <c r="G248" s="5" t="inlineStr">
         <is>
-          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+          <t>infra/launchd + scripts/ml_alert_slack.py</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr"/>
@@ -14327,18 +14327,18 @@
       </c>
       <c r="M248" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d1ea97913</t>
         </is>
       </c>
       <c r="N248" s="8" t="inlineStr"/>
     </row>
-    <row r="249" ht="75" customHeight="1">
+    <row r="249" ht="45" customHeight="1">
       <c r="A249" s="2" t="n">
         <v>248</v>
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
+          <t>FORENSICS-WEEKLY-SLACK</t>
         </is>
       </c>
       <c r="C249" s="10" t="inlineStr">
@@ -14348,39 +14348,27 @@
       </c>
       <c r="D249" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Notifications / Audit</t>
         </is>
       </c>
       <c r="E249" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Weekly pick-forensics Slack digest</t>
         </is>
       </c>
       <c r="F249" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
         </is>
       </c>
       <c r="G249" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
-        </is>
-      </c>
-      <c r="H249" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I249" s="5" t="inlineStr">
-        <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
-        </is>
-      </c>
-      <c r="J249" s="5" t="inlineStr">
-        <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
-        </is>
-      </c>
+          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr"/>
+      <c r="I249" s="5" t="inlineStr"/>
+      <c r="J249" s="5" t="inlineStr"/>
       <c r="K249" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14388,27 +14376,23 @@
       </c>
       <c r="L249" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M249" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N249" s="8" t="inlineStr">
-        <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="250" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N249" s="8" t="inlineStr"/>
+    </row>
+    <row r="250" ht="75" customHeight="1">
       <c r="A250" s="2" t="n">
         <v>249</v>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C250" s="10" t="inlineStr">
@@ -14418,37 +14402,37 @@
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E250" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F250" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G250" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I250" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J250" s="5" t="inlineStr">
         <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K250" s="12" t="inlineStr">
@@ -14458,17 +14442,17 @@
       </c>
       <c r="L250" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N250" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
         </is>
       </c>
     </row>
@@ -14478,7 +14462,7 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C251" s="10" t="inlineStr">
@@ -14493,32 +14477,32 @@
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F251" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G251" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I251" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J251" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K251" s="12" t="inlineStr">
@@ -14538,7 +14522,7 @@
       </c>
       <c r="N251" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -14548,7 +14532,7 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C252" s="10" t="inlineStr">
@@ -14563,32 +14547,32 @@
       </c>
       <c r="E252" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F252" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G252" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I252" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J252" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K252" s="12" t="inlineStr">
@@ -14608,7 +14592,7 @@
       </c>
       <c r="N252" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
         </is>
       </c>
     </row>
@@ -14618,7 +14602,7 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>OPS-4</t>
         </is>
       </c>
       <c r="C253" s="10" t="inlineStr">
@@ -14633,32 +14617,32 @@
       </c>
       <c r="E253" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F253" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G253" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I253" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J253" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K253" s="12" t="inlineStr">
@@ -14668,27 +14652,27 @@
       </c>
       <c r="L253" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M253" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N253" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="254" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="60" customHeight="1">
       <c r="A254" s="2" t="n">
         <v>253</v>
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>SCAN-FAILURE-ALERT</t>
+          <t>OPS-5</t>
         </is>
       </c>
       <c r="C254" s="10" t="inlineStr">
@@ -14698,27 +14682,39 @@
       </c>
       <c r="D254" s="5" t="inlineStr">
         <is>
-          <t>Ops / Alerts</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E254" s="6" t="inlineStr">
         <is>
-          <t>Scan-failure + EODHD-quota Slack alert</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F254" s="5" t="inlineStr">
         <is>
-          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G254" s="5" t="inlineStr">
         <is>
-          <t>swing_trade.py exit hook</t>
-        </is>
-      </c>
-      <c r="H254" s="2" t="inlineStr"/>
-      <c r="I254" s="5" t="inlineStr"/>
-      <c r="J254" s="5" t="inlineStr"/>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I254" s="5" t="inlineStr">
+        <is>
+          <t>Win: fast iteration on report templates.</t>
+        </is>
+      </c>
+      <c r="J254" s="5" t="inlineStr">
+        <is>
+          <t>Trivial CLI wrapper.</t>
+        </is>
+      </c>
       <c r="K254" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14726,15 +14722,19 @@
       </c>
       <c r="L254" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr">
         <is>
-          <t>0dc7675ee</t>
-        </is>
-      </c>
-      <c r="N254" s="8" t="inlineStr"/>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N254" s="8" t="inlineStr">
+        <is>
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="45" customHeight="1">
       <c r="A255" s="2" t="n">
@@ -14742,7 +14742,7 @@
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
+          <t>SCAN-FAILURE-ALERT</t>
         </is>
       </c>
       <c r="C255" s="10" t="inlineStr">
@@ -14752,22 +14752,22 @@
       </c>
       <c r="D255" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Alerts</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot: load or retire</t>
+          <t>Scan-failure + EODHD-quota Slack alert</t>
         </is>
       </c>
       <c r="F255" s="5" t="inlineStr">
         <is>
-          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
+          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
         </is>
       </c>
       <c r="G255" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd</t>
+          <t>swing_trade.py exit hook</t>
         </is>
       </c>
       <c r="H255" s="2" t="inlineStr"/>
@@ -14790,13 +14790,13 @@
       </c>
       <c r="N255" s="8" t="inlineStr"/>
     </row>
-    <row r="256" ht="60" customHeight="1">
+    <row r="256" ht="45" customHeight="1">
       <c r="A256" s="2" t="n">
         <v>255</v>
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>OVERVIEW-TQ-LABEL</t>
+          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
         </is>
       </c>
       <c r="C256" s="10" t="inlineStr">
@@ -14806,22 +14806,22 @@
       </c>
       <c r="D256" s="5" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E256" s="6" t="inlineStr">
         <is>
-          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
+          <t>Decide momentum-snapshot: load or retire</t>
         </is>
       </c>
       <c r="F256" s="5" t="inlineStr">
         <is>
-          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
+          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
         </is>
       </c>
       <c r="G256" s="5" t="inlineStr">
         <is>
-          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
+          <t>infra/launchd</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr"/>
@@ -14834,23 +14834,23 @@
       </c>
       <c r="L256" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M256" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>0dc7675ee</t>
         </is>
       </c>
       <c r="N256" s="8" t="inlineStr"/>
     </row>
-    <row r="257" ht="150" customHeight="1">
+    <row r="257" ht="60" customHeight="1">
       <c r="A257" s="2" t="n">
         <v>256</v>
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>OVERVIEW-TQ-LABEL</t>
         </is>
       </c>
       <c r="C257" s="10" t="inlineStr">
@@ -14860,31 +14860,27 @@
       </c>
       <c r="D257" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
         </is>
       </c>
       <c r="F257" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
         </is>
       </c>
       <c r="G257" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr"/>
       <c r="I257" s="5" t="inlineStr"/>
-      <c r="J257" s="5" t="inlineStr">
-        <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
-        </is>
-      </c>
+      <c r="J257" s="5" t="inlineStr"/>
       <c r="K257" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14892,27 +14888,23 @@
       </c>
       <c r="L257" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
-        </is>
-      </c>
-      <c r="N257" s="8" t="inlineStr">
-        <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="258" ht="105" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N257" s="8" t="inlineStr"/>
+    </row>
+    <row r="258" ht="150" customHeight="1">
       <c r="A258" s="2" t="n">
         <v>257</v>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>SMC-OB-DISPLAY-1</t>
+          <t>PERF-7b</t>
         </is>
       </c>
       <c r="C258" s="10" t="inlineStr">
@@ -14922,27 +14914,31 @@
       </c>
       <c r="D258" s="5" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E258" s="6" t="inlineStr">
         <is>
-          <t>OB confluence badges in SMC tab</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F258" s="5" t="inlineStr">
         <is>
-          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G258" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr"/>
       <c r="I258" s="5" t="inlineStr"/>
-      <c r="J258" s="5" t="inlineStr"/>
+      <c r="J258" s="5" t="inlineStr">
+        <is>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+        </is>
+      </c>
       <c r="K258" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14950,23 +14946,27 @@
       </c>
       <c r="L258" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr">
         <is>
-          <t>8182c3977</t>
-        </is>
-      </c>
-      <c r="N258" s="8" t="inlineStr"/>
-    </row>
-    <row r="259" ht="45" customHeight="1">
+          <t>cf30df858</t>
+        </is>
+      </c>
+      <c r="N258" s="8" t="inlineStr">
+        <is>
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="105" customHeight="1">
       <c r="A259" s="2" t="n">
         <v>258</v>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-1</t>
+          <t>SMC-OB-DISPLAY-1</t>
         </is>
       </c>
       <c r="C259" s="10" t="inlineStr">
@@ -14976,22 +14976,22 @@
       </c>
       <c r="D259" s="5" t="inlineStr">
         <is>
-          <t>Sharpe Roadmap</t>
+          <t>SMC</t>
         </is>
       </c>
       <c r="E259" s="6" t="inlineStr">
         <is>
-          <t>Sharpe gate in momentum detector</t>
+          <t>OB confluence badges in SMC tab</t>
         </is>
       </c>
       <c r="F259" s="5" t="inlineStr">
         <is>
-          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
+          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
         </is>
       </c>
       <c r="G259" s="5" t="inlineStr">
         <is>
-          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
+          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr"/>
@@ -15004,12 +15004,12 @@
       </c>
       <c r="L259" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr">
         <is>
-          <t>dbbd6b5f6</t>
+          <t>8182c3977</t>
         </is>
       </c>
       <c r="N259" s="8" t="inlineStr"/>
@@ -15020,7 +15020,7 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-10</t>
+          <t>SHARPE-1</t>
         </is>
       </c>
       <c r="C260" s="10" t="inlineStr">
@@ -15035,17 +15035,17 @@
       </c>
       <c r="E260" s="6" t="inlineStr">
         <is>
-          <t>Sharpe alerts for watchlist</t>
+          <t>Sharpe gate in momentum detector</t>
         </is>
       </c>
       <c r="F260" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
         </is>
       </c>
       <c r="G260" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
+          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr"/>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-11</t>
+          <t>SHARPE-10</t>
         </is>
       </c>
       <c r="C261" s="10" t="inlineStr">
@@ -15089,17 +15089,17 @@
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>Per-trade Sharpe attribution</t>
+          <t>Sharpe alerts for watchlist</t>
         </is>
       </c>
       <c r="F261" s="5" t="inlineStr">
         <is>
-          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G261" s="5" t="inlineStr">
         <is>
-          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
+          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr"/>
@@ -15128,7 +15128,7 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-12</t>
+          <t>SHARPE-11</t>
         </is>
       </c>
       <c r="C262" s="10" t="inlineStr">
@@ -15143,17 +15143,17 @@
       </c>
       <c r="E262" s="6" t="inlineStr">
         <is>
-          <t>Sharpe consistency check</t>
+          <t>Per-trade Sharpe attribution</t>
         </is>
       </c>
       <c r="F262" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
         </is>
       </c>
       <c r="G262" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
+          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr"/>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-2</t>
+          <t>SHARPE-12</t>
         </is>
       </c>
       <c r="C263" s="10" t="inlineStr">
@@ -15197,17 +15197,17 @@
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>Sharpe column in v2 dashboard</t>
+          <t>Sharpe consistency check</t>
         </is>
       </c>
       <c r="F263" s="5" t="inlineStr">
         <is>
-          <t>Surface 126d Sharpe per ticker as sortable column</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G263" s="5" t="inlineStr">
         <is>
-          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
+          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr"/>
@@ -15236,7 +15236,7 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-3</t>
+          <t>SHARPE-2</t>
         </is>
       </c>
       <c r="C264" s="10" t="inlineStr">
@@ -15251,17 +15251,17 @@
       </c>
       <c r="E264" s="6" t="inlineStr">
         <is>
-          <t>Per-stock Sharpe by regime</t>
+          <t>Sharpe column in v2 dashboard</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
         <is>
-          <t>Decompose per-stock Sharpe by historical regime tags</t>
+          <t>Surface 126d Sharpe per ticker as sortable column</t>
         </is>
       </c>
       <c r="G264" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
+          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr"/>
@@ -15290,7 +15290,7 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-4</t>
+          <t>SHARPE-3</t>
         </is>
       </c>
       <c r="C265" s="10" t="inlineStr">
@@ -15305,17 +15305,17 @@
       </c>
       <c r="E265" s="6" t="inlineStr">
         <is>
-          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
+          <t>Per-stock Sharpe by regime</t>
         </is>
       </c>
       <c r="F265" s="5" t="inlineStr">
         <is>
-          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
+          <t>Decompose per-stock Sharpe by historical regime tags</t>
         </is>
       </c>
       <c r="G265" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
+          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr"/>
@@ -15344,7 +15344,7 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-5</t>
+          <t>SHARPE-4</t>
         </is>
       </c>
       <c r="C266" s="10" t="inlineStr">
@@ -15359,17 +15359,17 @@
       </c>
       <c r="E266" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-weighted position sizing</t>
+          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
         </is>
       </c>
       <c r="F266" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
         </is>
       </c>
       <c r="G266" s="5" t="inlineStr">
         <is>
-          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr"/>
@@ -15398,7 +15398,7 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-6</t>
+          <t>SHARPE-5</t>
         </is>
       </c>
       <c r="C267" s="10" t="inlineStr">
@@ -15413,17 +15413,17 @@
       </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>Portfolio Sharpe KPI vs target</t>
+          <t>Sharpe-weighted position sizing</t>
         </is>
       </c>
       <c r="F267" s="5" t="inlineStr">
         <is>
-          <t>Annualized Sharpe target tracking + gap report</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G267" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
+          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr"/>
@@ -15452,7 +15452,7 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-7</t>
+          <t>SHARPE-6</t>
         </is>
       </c>
       <c r="C268" s="10" t="inlineStr">
@@ -15467,17 +15467,17 @@
       </c>
       <c r="E268" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-based stop sizing</t>
+          <t>Portfolio Sharpe KPI vs target</t>
         </is>
       </c>
       <c r="F268" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Annualized Sharpe target tracking + gap report</t>
         </is>
       </c>
       <c r="G268" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr"/>
@@ -15506,7 +15506,7 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-8</t>
+          <t>SHARPE-7</t>
         </is>
       </c>
       <c r="C269" s="10" t="inlineStr">
@@ -15521,17 +15521,17 @@
       </c>
       <c r="E269" s="6" t="inlineStr">
         <is>
-          <t>Sortino computation alongside Sharpe</t>
+          <t>Sharpe-based stop sizing</t>
         </is>
       </c>
       <c r="F269" s="5" t="inlineStr">
         <is>
-          <t>Downside-only vol denominator added everywhere</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G269" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
+          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H269" s="2" t="inlineStr"/>
@@ -15560,7 +15560,7 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-9</t>
+          <t>SHARPE-8</t>
         </is>
       </c>
       <c r="C270" s="10" t="inlineStr">
@@ -15575,17 +15575,17 @@
       </c>
       <c r="E270" s="6" t="inlineStr">
         <is>
-          <t>SPY-Sharpe regime cross-validation</t>
+          <t>Sortino computation alongside Sharpe</t>
         </is>
       </c>
       <c r="F270" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Downside-only vol denominator added everywhere</t>
         </is>
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
+          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr"/>
@@ -15608,13 +15608,13 @@
       </c>
       <c r="N270" s="8" t="inlineStr"/>
     </row>
-    <row r="271" ht="60" customHeight="1">
+    <row r="271" ht="45" customHeight="1">
       <c r="A271" s="2" t="n">
         <v>270</v>
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-RECUR-CHIP</t>
+          <t>SHARPE-9</t>
         </is>
       </c>
       <c r="C271" s="10" t="inlineStr">
@@ -15624,22 +15624,22 @@
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>Signal Scanner</t>
+          <t>Sharpe Roadmap</t>
         </is>
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>Recurrence chip</t>
+          <t>SPY-Sharpe regime cross-validation</t>
         </is>
       </c>
       <c r="F271" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr"/>
@@ -15652,23 +15652,23 @@
       </c>
       <c r="L271" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M271" s="3" t="inlineStr">
         <is>
-          <t>cf702f2b4</t>
+          <t>dbbd6b5f6</t>
         </is>
       </c>
       <c r="N271" s="8" t="inlineStr"/>
     </row>
-    <row r="272" ht="120" customHeight="1">
+    <row r="272" ht="60" customHeight="1">
       <c r="A272" s="2" t="n">
         <v>271</v>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>CONVICTION-TIER-WIRE</t>
+          <t>SCANNER-RECUR-CHIP</t>
         </is>
       </c>
       <c r="C272" s="10" t="inlineStr">
@@ -15678,39 +15678,27 @@
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Conviction</t>
+          <t>Signal Scanner</t>
         </is>
       </c>
       <c r="E272" s="6" t="inlineStr">
         <is>
-          <t>Conviction tier: simplified to score-band only</t>
+          <t>Recurrence chip</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
         <is>
-          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
+          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
         </is>
       </c>
       <c r="G272" s="5" t="inlineStr">
         <is>
-          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
-        </is>
-      </c>
-      <c r="H272" s="2" t="inlineStr">
-        <is>
-          <t>2-4 hrs + backtest validation</t>
-        </is>
-      </c>
-      <c r="I272" s="5" t="inlineStr">
-        <is>
-          <t>Medium — changes live size or eliminates a layer</t>
-        </is>
-      </c>
-      <c r="J272" s="5" t="inlineStr">
-        <is>
-          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
-        </is>
-      </c>
+          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr"/>
+      <c r="I272" s="5" t="inlineStr"/>
+      <c r="J272" s="5" t="inlineStr"/>
       <c r="K272" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15718,27 +15706,23 @@
       </c>
       <c r="L272" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M272" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N272" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
-        </is>
-      </c>
-    </row>
-    <row r="273" ht="75" customHeight="1">
+          <t>cf702f2b4</t>
+        </is>
+      </c>
+      <c r="N272" s="8" t="inlineStr"/>
+    </row>
+    <row r="273" ht="120" customHeight="1">
       <c r="A273" s="2" t="n">
         <v>272</v>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-Q-AB</t>
+          <t>CONVICTION-TIER-WIRE</t>
         </is>
       </c>
       <c r="C273" s="10" t="inlineStr">
@@ -15748,27 +15732,39 @@
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Gates</t>
+          <t>Strategy / Conviction</t>
         </is>
       </c>
       <c r="E273" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional entry_quality A/B</t>
+          <t>Conviction tier: simplified to score-band only</t>
         </is>
       </c>
       <c r="F273" s="5" t="inlineStr">
         <is>
-          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
+          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
         </is>
       </c>
       <c r="G273" s="5" t="inlineStr">
         <is>
-          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
-        </is>
-      </c>
-      <c r="H273" s="2" t="inlineStr"/>
-      <c r="I273" s="5" t="inlineStr"/>
-      <c r="J273" s="5" t="inlineStr"/>
+          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>2-4 hrs + backtest validation</t>
+        </is>
+      </c>
+      <c r="I273" s="5" t="inlineStr">
+        <is>
+          <t>Medium — changes live size or eliminates a layer</t>
+        </is>
+      </c>
+      <c r="J273" s="5" t="inlineStr">
+        <is>
+          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
+        </is>
+      </c>
       <c r="K273" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15776,23 +15772,27 @@
       </c>
       <c r="L273" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr">
         <is>
-          <t>07c3af6a3</t>
-        </is>
-      </c>
-      <c r="N273" s="8" t="inlineStr"/>
-    </row>
-    <row r="274" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N273" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="75" customHeight="1">
       <c r="A274" s="2" t="n">
         <v>273</v>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-1</t>
+          <t>ENTRY-Q-AB</t>
         </is>
       </c>
       <c r="C274" s="10" t="inlineStr">
@@ -15802,22 +15802,22 @@
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Options Paper</t>
+          <t>Strategy / Gates</t>
         </is>
       </c>
       <c r="E274" s="6" t="inlineStr">
         <is>
-          <t>Signal -&gt; options-structure mapper</t>
+          <t>Regime-conditional entry_quality A/B</t>
         </is>
       </c>
       <c r="F274" s="5" t="inlineStr">
         <is>
-          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
+          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
         </is>
       </c>
       <c r="G274" s="5" t="inlineStr">
         <is>
-          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
+          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr"/>
@@ -15830,23 +15830,23 @@
       </c>
       <c r="L274" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr">
         <is>
-          <t>9c3a2a58d</t>
+          <t>07c3af6a3</t>
         </is>
       </c>
       <c r="N274" s="8" t="inlineStr"/>
     </row>
-    <row r="275" ht="45" customHeight="1">
+    <row r="275" ht="60" customHeight="1">
       <c r="A275" s="2" t="n">
         <v>274</v>
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-2</t>
+          <t>OPT-PAPER-1</t>
         </is>
       </c>
       <c r="C275" s="10" t="inlineStr">
@@ -15861,17 +15861,17 @@
       </c>
       <c r="E275" s="6" t="inlineStr">
         <is>
-          <t>Contract selection from Schwab chain</t>
+          <t>Signal -&gt; options-structure mapper</t>
         </is>
       </c>
       <c r="F275" s="5" t="inlineStr">
         <is>
-          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
+          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
         </is>
       </c>
       <c r="G275" s="5" t="inlineStr">
         <is>
-          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
+          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr"/>
@@ -15894,13 +15894,13 @@
       </c>
       <c r="N275" s="8" t="inlineStr"/>
     </row>
-    <row r="276" ht="60" customHeight="1">
+    <row r="276" ht="45" customHeight="1">
       <c r="A276" s="2" t="n">
         <v>275</v>
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-3</t>
+          <t>OPT-PAPER-2</t>
         </is>
       </c>
       <c r="C276" s="10" t="inlineStr">
@@ -15915,17 +15915,17 @@
       </c>
       <c r="E276" s="6" t="inlineStr">
         <is>
-          <t>Alpaca paper options orders in executor.py</t>
+          <t>Contract selection from Schwab chain</t>
         </is>
       </c>
       <c r="F276" s="5" t="inlineStr">
         <is>
-          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
+          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
         </is>
       </c>
       <c r="G276" s="5" t="inlineStr">
         <is>
-          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
+          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr"/>
@@ -15948,13 +15948,13 @@
       </c>
       <c r="N276" s="8" t="inlineStr"/>
     </row>
-    <row r="277" ht="45" customHeight="1">
+    <row r="277" ht="60" customHeight="1">
       <c r="A277" s="2" t="n">
         <v>276</v>
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-4</t>
+          <t>OPT-PAPER-3</t>
         </is>
       </c>
       <c r="C277" s="10" t="inlineStr">
@@ -15969,17 +15969,17 @@
       </c>
       <c r="E277" s="6" t="inlineStr">
         <is>
-          <t>Options position tracking + contract P&amp;L</t>
+          <t>Alpaca paper options orders in executor.py</t>
         </is>
       </c>
       <c r="F277" s="5" t="inlineStr">
         <is>
-          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
+          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
         </is>
       </c>
       <c r="G277" s="5" t="inlineStr">
         <is>
-          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
+          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr"/>
@@ -15997,7 +15997,7 @@
       </c>
       <c r="M277" s="3" t="inlineStr">
         <is>
-          <t>635ae960f</t>
+          <t>9c3a2a58d</t>
         </is>
       </c>
       <c r="N277" s="8" t="inlineStr"/>
@@ -16008,7 +16008,7 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-5</t>
+          <t>OPT-PAPER-4</t>
         </is>
       </c>
       <c r="C278" s="10" t="inlineStr">
@@ -16023,17 +16023,17 @@
       </c>
       <c r="E278" s="6" t="inlineStr">
         <is>
-          <t>Options-specific exits</t>
+          <t>Options position tracking + contract P&amp;L</t>
         </is>
       </c>
       <c r="F278" s="5" t="inlineStr">
         <is>
-          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
+          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
         </is>
       </c>
       <c r="G278" s="5" t="inlineStr">
         <is>
-          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
+          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr"/>
@@ -16056,13 +16056,13 @@
       </c>
       <c r="N278" s="8" t="inlineStr"/>
     </row>
-    <row r="279" ht="120" customHeight="1">
+    <row r="279" ht="45" customHeight="1">
       <c r="A279" s="2" t="n">
         <v>278</v>
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>UI-STRAT-1</t>
+          <t>OPT-PAPER-5</t>
         </is>
       </c>
       <c r="C279" s="10" t="inlineStr">
@@ -16072,22 +16072,22 @@
       </c>
       <c r="D279" s="5" t="inlineStr">
         <is>
-          <t>Strategy Lab</t>
+          <t>Strategy / Options Paper</t>
         </is>
       </c>
       <c r="E279" s="6" t="inlineStr">
         <is>
-          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
+          <t>Options-specific exits</t>
         </is>
       </c>
       <c r="F279" s="5" t="inlineStr">
         <is>
-          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
+          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
         </is>
       </c>
       <c r="G279" s="5" t="inlineStr">
         <is>
-          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
+          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr"/>
@@ -16100,23 +16100,23 @@
       </c>
       <c r="L279" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="M279" s="3" t="inlineStr">
         <is>
-          <t>93ec11842</t>
+          <t>635ae960f</t>
         </is>
       </c>
       <c r="N279" s="8" t="inlineStr"/>
     </row>
-    <row r="280" ht="60" customHeight="1">
+    <row r="280" ht="120" customHeight="1">
       <c r="A280" s="2" t="n">
         <v>279</v>
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>TE-STRATEGY-MODE</t>
+          <t>UI-STRAT-1</t>
         </is>
       </c>
       <c r="C280" s="10" t="inlineStr">
@@ -16126,22 +16126,22 @@
       </c>
       <c r="D280" s="5" t="inlineStr">
         <is>
-          <t>Target Engine</t>
+          <t>Strategy Lab</t>
         </is>
       </c>
       <c r="E280" s="6" t="inlineStr">
         <is>
-          <t>_strategy_mode read but never written</t>
+          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
+          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
         </is>
       </c>
       <c r="G280" s="5" t="inlineStr">
         <is>
-          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
+          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr"/>
@@ -16154,23 +16154,23 @@
       </c>
       <c r="L280" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>93ec11842</t>
         </is>
       </c>
       <c r="N280" s="8" t="inlineStr"/>
     </row>
-    <row r="281" ht="105" customHeight="1">
+    <row r="281" ht="60" customHeight="1">
       <c r="A281" s="2" t="n">
         <v>280</v>
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>TRACKER-BUY-FILTER</t>
+          <t>TE-STRATEGY-MODE</t>
         </is>
       </c>
       <c r="C281" s="10" t="inlineStr">
@@ -16180,31 +16180,27 @@
       </c>
       <c r="D281" s="5" t="inlineStr">
         <is>
-          <t>Tracker/Feedback Loop</t>
+          <t>Target Engine</t>
         </is>
       </c>
       <c r="E281" s="6" t="inlineStr">
         <is>
-          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
+          <t>_strategy_mode read but never written</t>
         </is>
       </c>
       <c r="F281" s="5" t="inlineStr">
         <is>
-          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
+          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
         </is>
       </c>
       <c r="G281" s="5" t="inlineStr">
         <is>
-          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr"/>
       <c r="I281" s="5" t="inlineStr"/>
-      <c r="J281" s="5" t="inlineStr">
-        <is>
-          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
-        </is>
-      </c>
+      <c r="J281" s="5" t="inlineStr"/>
       <c r="K281" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16212,27 +16208,23 @@
       </c>
       <c r="L281" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N281" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="282" ht="135" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N281" s="8" t="inlineStr"/>
+    </row>
+    <row r="282" ht="105" customHeight="1">
       <c r="A282" s="2" t="n">
         <v>281</v>
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
+          <t>TRACKER-BUY-FILTER</t>
         </is>
       </c>
       <c r="C282" s="10" t="inlineStr">
@@ -16242,37 +16234,29 @@
       </c>
       <c r="D282" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Tracker/Feedback Loop</t>
         </is>
       </c>
       <c r="E282" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
         </is>
       </c>
       <c r="G282" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
-        </is>
-      </c>
-      <c r="H282" s="2" t="inlineStr">
-        <is>
-          <t>1-2 hrs</t>
-        </is>
-      </c>
-      <c r="I282" s="5" t="inlineStr">
-        <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
-        </is>
-      </c>
+          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr"/>
+      <c r="I282" s="5" t="inlineStr"/>
       <c r="J282" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
         </is>
       </c>
       <c r="K282" s="12" t="inlineStr">
@@ -16282,27 +16266,27 @@
       </c>
       <c r="L282" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr">
         <is>
-          <t>42c36ef91</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N282" s="8" t="inlineStr">
         <is>
-          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="283" ht="45" customHeight="1">
+          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="135" customHeight="1">
       <c r="A283" s="2" t="n">
         <v>282</v>
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>STOCKSMITH-BOOK-RISK</t>
+          <t>MOD-1</t>
         </is>
       </c>
       <c r="C283" s="10" t="inlineStr">
@@ -16312,27 +16296,39 @@
       </c>
       <c r="D283" s="5" t="inlineStr">
         <is>
-          <t>V2 Dashboard / Risk</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E283" s="6" t="inlineStr">
         <is>
-          <t>Book Risk surface + per-lens analytics (§6)</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G283" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
-        </is>
-      </c>
-      <c r="H283" s="2" t="inlineStr"/>
-      <c r="I283" s="5" t="inlineStr"/>
-      <c r="J283" s="5" t="inlineStr"/>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I283" s="5" t="inlineStr">
+        <is>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
+        </is>
+      </c>
+      <c r="J283" s="5" t="inlineStr">
+        <is>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+        </is>
+      </c>
       <c r="K283" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16340,23 +16336,27 @@
       </c>
       <c r="L283" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr">
         <is>
-          <t>50cace567</t>
-        </is>
-      </c>
-      <c r="N283" s="8" t="inlineStr"/>
-    </row>
-    <row r="284" ht="120" customHeight="1">
+          <t>42c36ef91</t>
+        </is>
+      </c>
+      <c r="N283" s="8" t="inlineStr">
+        <is>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="45" customHeight="1">
       <c r="A284" s="2" t="n">
         <v>283</v>
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>RECENCY-FLOOR</t>
+          <t>STOCKSMITH-BOOK-RISK</t>
         </is>
       </c>
       <c r="C284" s="10" t="inlineStr">
@@ -16366,31 +16366,27 @@
       </c>
       <c r="D284" s="5" t="inlineStr">
         <is>
-          <t>Validation Hygiene</t>
+          <t>V2 Dashboard / Risk</t>
         </is>
       </c>
       <c r="E284" s="6" t="inlineStr">
         <is>
-          <t>_validations needs recency floor — auto-revert stale boosts</t>
+          <t>Book Risk surface + per-lens analytics (§6)</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
+          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
         </is>
       </c>
       <c r="G284" s="5" t="inlineStr">
         <is>
-          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
+          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr"/>
       <c r="I284" s="5" t="inlineStr"/>
-      <c r="J284" s="5" t="inlineStr">
-        <is>
-          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
-        </is>
-      </c>
+      <c r="J284" s="5" t="inlineStr"/>
       <c r="K284" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16398,27 +16394,23 @@
       </c>
       <c r="L284" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N284" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="285" ht="60" customHeight="1">
+          <t>50cace567</t>
+        </is>
+      </c>
+      <c r="N284" s="8" t="inlineStr"/>
+    </row>
+    <row r="285" ht="120" customHeight="1">
       <c r="A285" s="2" t="n">
         <v>284</v>
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-TAB</t>
+          <t>RECENCY-FLOOR</t>
         </is>
       </c>
       <c r="C285" s="10" t="inlineStr">
@@ -16428,27 +16420,31 @@
       </c>
       <c r="D285" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Momentum</t>
+          <t>Validation Hygiene</t>
         </is>
       </c>
       <c r="E285" s="6" t="inlineStr">
         <is>
-          <t>New 🚀 Momentum workspace tab</t>
+          <t>_validations needs recency floor — auto-revert stale boosts</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
+          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
         </is>
       </c>
       <c r="G285" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
+          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr"/>
       <c r="I285" s="5" t="inlineStr"/>
-      <c r="J285" s="5" t="inlineStr"/>
+      <c r="J285" s="5" t="inlineStr">
+        <is>
+          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
+        </is>
+      </c>
       <c r="K285" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16456,15 +16452,19 @@
       </c>
       <c r="L285" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N285" s="8" t="inlineStr"/>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N285" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
+        </is>
+      </c>
     </row>
     <row r="286" ht="60" customHeight="1">
       <c r="A286" s="2" t="n">
@@ -16472,7 +16472,7 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-QUICK-PANELS</t>
+          <t>MOMENTUM-TAB</t>
         </is>
       </c>
       <c r="C286" s="10" t="inlineStr">
@@ -16482,22 +16482,22 @@
       </c>
       <c r="D286" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Signal Scanner</t>
+          <t>Workspaces / Momentum</t>
         </is>
       </c>
       <c r="E286" s="6" t="inlineStr">
         <is>
-          <t>5 quick-glance panels above watchlist table</t>
+          <t>New 🚀 Momentum workspace tab</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
+          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
         </is>
       </c>
       <c r="G286" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr"/>
@@ -16515,60 +16515,48 @@
       </c>
       <c r="M286" s="3" t="inlineStr">
         <is>
-          <t>dfbe955fe</t>
+          <t>27fd646b1</t>
         </is>
       </c>
       <c r="N286" s="8" t="inlineStr"/>
     </row>
-    <row r="287" ht="45" customHeight="1">
+    <row r="287" ht="60" customHeight="1">
       <c r="A287" s="2" t="n">
         <v>286</v>
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C287" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>SCANNER-QUICK-PANELS</t>
+        </is>
+      </c>
+      <c r="C287" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Workspaces / Signal Scanner</t>
         </is>
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>5 quick-glance panels above watchlist table</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
         </is>
       </c>
       <c r="G287" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
-        </is>
-      </c>
-      <c r="H287" s="2" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="I287" s="5" t="inlineStr">
-        <is>
-          <t>Win: persistence works; no silent overwrites.</t>
-        </is>
-      </c>
-      <c r="J287" s="5" t="inlineStr">
-        <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
-        </is>
-      </c>
+          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr"/>
+      <c r="I287" s="5" t="inlineStr"/>
+      <c r="J287" s="5" t="inlineStr"/>
       <c r="K287" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16576,15 +16564,15 @@
       </c>
       <c r="L287" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M287" s="3" t="inlineStr"/>
-      <c r="N287" s="8" t="inlineStr">
-        <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="M287" s="3" t="inlineStr">
+        <is>
+          <t>dfbe955fe</t>
+        </is>
+      </c>
+      <c r="N287" s="8" t="inlineStr"/>
     </row>
     <row r="288" ht="45" customHeight="1">
       <c r="A288" s="2" t="n">
@@ -16592,7 +16580,7 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="C288" s="13" t="inlineStr">
@@ -16607,32 +16595,32 @@
       </c>
       <c r="E288" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G288" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
-          <t>verified (no change needed)</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I288" s="5" t="inlineStr">
         <is>
-          <t>Win: confirms infrastructure still healthy.</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J288" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
         </is>
       </c>
       <c r="K288" s="12" t="inlineStr">
@@ -16648,7 +16636,7 @@
       <c r="M288" s="3" t="inlineStr"/>
       <c r="N288" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
         </is>
       </c>
     </row>
@@ -16658,7 +16646,7 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>UI-3</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -16668,35 +16656,39 @@
       </c>
       <c r="D289" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E289" s="6" t="inlineStr">
         <is>
-          <t>Remove emoji icons from Thesis + Research labels</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G289" s="5" t="inlineStr">
         <is>
-          <t>Removed emojis from FD sub-tab nav + section headers.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I289" s="5" t="inlineStr">
         <is>
-          <t>Low / cosmetic</t>
-        </is>
-      </c>
-      <c r="J289" s="5" t="inlineStr"/>
+          <t>Win: confirms infrastructure still healthy.</t>
+        </is>
+      </c>
+      <c r="J289" s="5" t="inlineStr">
+        <is>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
       <c r="K289" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16704,17 +16696,13 @@
       </c>
       <c r="L289" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="M289" s="3" t="inlineStr">
-        <is>
-          <t>24fd7c273</t>
-        </is>
-      </c>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M289" s="3" t="inlineStr"/>
       <c r="N289" s="8" t="inlineStr">
         <is>
-          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
         </is>
       </c>
     </row>
@@ -16724,59 +16712,63 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
-        </is>
-      </c>
-      <c r="C290" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>UI-3</t>
+        </is>
+      </c>
+      <c r="C290" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D290" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Remove emoji icons from Thesis + Research labels</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
         </is>
       </c>
       <c r="G290" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+          <t>Removed emojis from FD sub-tab nav + section headers.</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>5 min after answer</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I290" s="5" t="inlineStr">
         <is>
-          <t>Win: -671 lines.</t>
-        </is>
-      </c>
-      <c r="J290" s="5" t="inlineStr">
-        <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K290" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L290" s="2" t="inlineStr"/>
-      <c r="M290" s="3" t="inlineStr"/>
+          <t>Low / cosmetic</t>
+        </is>
+      </c>
+      <c r="J290" s="5" t="inlineStr"/>
+      <c r="K290" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L290" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M290" s="3" t="inlineStr">
+        <is>
+          <t>24fd7c273</t>
+        </is>
+      </c>
       <c r="N290" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
         </is>
       </c>
     </row>
@@ -16786,7 +16778,7 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
+          <t>CLEAN-2</t>
         </is>
       </c>
       <c r="C291" s="10" t="inlineStr">
@@ -16796,37 +16788,37 @@
       </c>
       <c r="D291" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E291" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
         </is>
       </c>
       <c r="G291" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>5 min after answer</t>
         </is>
       </c>
       <c r="I291" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Win: -671 lines.</t>
         </is>
       </c>
       <c r="J291" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
+          <t>Standard data-migration retention practice.</t>
         </is>
       </c>
       <c r="K291" s="14" t="inlineStr">
@@ -16848,109 +16840,109 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C292" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C292" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D292" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E292" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
         </is>
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
         </is>
       </c>
       <c r="G292" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>hours-days each</t>
         </is>
       </c>
       <c r="I292" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win varies; defer until PERF-7 measured.</t>
         </is>
       </c>
       <c r="J292" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K292" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K292" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="L292" s="2" t="inlineStr"/>
       <c r="M292" s="3" t="inlineStr"/>
       <c r="N292" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="293" ht="75" customHeight="1">
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="45" customHeight="1">
       <c r="A293" s="2" t="n">
         <v>292</v>
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>MOD-2</t>
-        </is>
-      </c>
-      <c r="C293" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C293" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D293" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E293" s="6" t="inlineStr">
         <is>
-          <t>Pixel-diff regression baseline</t>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>After modularization, no automated visual-regression catch.</t>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
         </is>
       </c>
       <c r="G293" s="5" t="inlineStr">
         <is>
-          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
         </is>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I293" s="5" t="inlineStr">
         <is>
-          <t>Win: catches accidental layout regressions.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J293" s="5" t="inlineStr">
         <is>
-          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+          <t>Agents skim and miss post-filter subset analysis.</t>
         </is>
       </c>
       <c r="K293" s="15" t="inlineStr">
@@ -16958,147 +16950,209 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L293" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
+      <c r="L293" s="2" t="inlineStr"/>
       <c r="M293" s="3" t="inlineStr"/>
       <c r="N293" s="8" t="inlineStr">
         <is>
-          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="294" ht="195" customHeight="1">
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="75" customHeight="1">
       <c r="A294" s="2" t="n">
         <v>293</v>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
+          <t>MOD-2</t>
+        </is>
+      </c>
+      <c r="C294" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D294" s="5" t="inlineStr">
+        <is>
+          <t>UI / Modularization</t>
+        </is>
+      </c>
+      <c r="E294" s="6" t="inlineStr">
+        <is>
+          <t>Pixel-diff regression baseline</t>
+        </is>
+      </c>
+      <c r="F294" s="5" t="inlineStr">
+        <is>
+          <t>After modularization, no automated visual-regression catch.</t>
+        </is>
+      </c>
+      <c r="G294" s="5" t="inlineStr">
+        <is>
+          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+        </is>
+      </c>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t>2-3 hrs</t>
+        </is>
+      </c>
+      <c r="I294" s="5" t="inlineStr">
+        <is>
+          <t>Win: catches accidental layout regressions.</t>
+        </is>
+      </c>
+      <c r="J294" s="5" t="inlineStr">
+        <is>
+          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+        </is>
+      </c>
+      <c r="K294" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L294" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="M294" s="3" t="inlineStr"/>
+      <c r="N294" s="8" t="inlineStr">
+        <is>
+          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="195" customHeight="1">
+      <c r="A295" s="2" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
           <t>OB-CONFLUENCE-PROPOSAL-REJECTED</t>
         </is>
       </c>
-      <c r="C294" s="10" t="inlineStr">
+      <c r="C295" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D294" s="5" t="inlineStr">
+      <c r="D295" s="5" t="inlineStr">
         <is>
           <t>Signals / Cross-Check</t>
         </is>
       </c>
-      <c r="E294" s="6" t="inlineStr">
+      <c r="E295" s="6" t="inlineStr">
         <is>
           <t>OB-confluence Wilson bump + OB-aware stop — proposals KILLED by backtest evidence</t>
         </is>
       </c>
-      <c r="F294" s="5" t="inlineStr">
+      <c r="F295" s="5" t="inlineStr">
         <is>
           <t>User asked 2026-05-12 to ship #2 (Wilson-bump score factor for bullish OB confluence within 5% of entry) and #5 (OB-low as stop instead of 1.25xATR). Per Principle 1 / Principle 7, ran post-hoc validation: scripts/validate_ob_confluence.py retroactively tags every closed trade from existing portfolio_backtest outputs with SMC state at entry date, computes Wilson 95% LB per subset.
 RESULT (750-day backtest · n=384): Bull OB confluence within 5% of entry DECREASES Wilson LB by -8.6pp (14.6% vs baseline 23.1%). BOS-bullish boost: -3.4pp. SMC-bullish direction boost: -3.6pp. Per #5 simulation, 35 of 39 (90%) OB-low-as-stop would have loosened the stop; 25 of those still ended in losses (looser stops do not rescue broken setups, they extend exposure).
 Principle 4 fires: proposals FALSIFIED, killed permanently (not retuned). Doing the change without this validation would have introduced a 6-9pp Wilson-LB drag on every BUY signal.</t>
         </is>
       </c>
-      <c r="G294" s="5" t="inlineStr">
+      <c r="G295" s="5" t="inlineStr">
         <is>
           <t>Built scripts/validate_ob_confluence.py to retroactively run smart_money.score_smc() on the historical OHLCV at each trade's entry date, tag with OB-confluence + BOS + CHoCH flags, compute Wilson 95% LB per subset, and apply Principle 1 gates (n&gt;=30, lift&gt;=5pp). Cross-validated on 250d (n=142) and 750d (n=384) backtest outputs. Both agree: NO EDGE.</t>
         </is>
       </c>
-      <c r="H294" s="2" t="inlineStr">
+      <c r="H295" s="2" t="inlineStr">
         <is>
           <t>Days of work avoided (would have shipped a degrading change).</t>
         </is>
       </c>
-      <c r="I294" s="5" t="inlineStr">
+      <c r="I295" s="5" t="inlineStr">
         <is>
           <t>Mechanism (Principle 2): institutional OBs are supposed to mark re-add zones for smart money. Falsification (Principle 4): if the data doesn't show OB-confluent trades winning more, the mechanism either doesn't exist for retail-accessible OB detection at daily resolution OR is already priced into our 5-pillar score. Either way: ship nothing. The proposals are dead. Win: prevented a 6-9pp Wilson-LB drag from being added to live scoring. Lost: nothing — we didn't change live scoring, no opportunity cost.</t>
         </is>
       </c>
-      <c r="J294" s="5" t="inlineStr">
+      <c r="J295" s="5" t="inlineStr">
         <is>
           <t>Validator script is reusable infrastructure. Re-run any time the SMC detection logic or score thresholds change. NOTE: baseline WR in 750d backtest is 27.3% (low) — the absolute level reflects backtest-window-specific market conditions; the SUBSET comparisons are valid regardless because they share the same baseline. Do not interpret 23.1% Wilson LB as a system-level edge — that's a separate question. This validation answers ONLY: does OB-confluence improve selection within whatever the system already does.</t>
         </is>
       </c>
-      <c r="K294" s="15" t="inlineStr">
+      <c r="K295" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L294" s="2" t="inlineStr">
+      <c r="L295" s="2" t="inlineStr">
         <is>
           <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="M294" s="3" t="inlineStr"/>
-      <c r="N294" s="8" t="inlineStr">
-        <is>
-          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="295" ht="90" customHeight="1">
-      <c r="A295" s="2" t="n">
-        <v>294</v>
-      </c>
-      <c r="B295" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C295" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="D295" s="5" t="inlineStr">
-        <is>
-          <t>Data / Universe</t>
-        </is>
-      </c>
-      <c r="E295" s="6" t="inlineStr">
-        <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
-        </is>
-      </c>
-      <c r="F295" s="5" t="inlineStr">
-        <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
-        </is>
-      </c>
-      <c r="G295" s="5" t="inlineStr">
-        <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
-        </is>
-      </c>
-      <c r="H295" s="2" t="inlineStr">
-        <is>
-          <t>$$ + 1 day</t>
-        </is>
-      </c>
-      <c r="I295" s="5" t="inlineStr">
-        <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
-        </is>
-      </c>
-      <c r="J295" s="5" t="inlineStr">
-        <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K295" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L295" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M295" s="3" t="inlineStr"/>
       <c r="N295" s="8" t="inlineStr">
+        <is>
+          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="90" customHeight="1">
+      <c r="A296" s="2" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C296" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D296" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E296" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F296" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G296" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I296" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J296" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K296" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L296" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M296" s="3" t="inlineStr"/>
+      <c r="N296" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -17203,10 +17257,10 @@
         <v>86</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5">
@@ -17260,10 +17314,10 @@
         <v>111</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FEAT: dedicated catalyst-sleeve signal alerts (PEAD/Insider/ESP/...) — SLEEVE-ALERTS
The entry-watcher covers price-action setups (pullback/breakout/impulse) but the
7 catalyst sleeves had no dedicated alert — they only surfaced indirectly via the
flip/elite digests. These are the higher-mechanism signals (principle 14; PEAD
backtested PF 2.04, Momentum 1.53), so they warrant a direct ping. signal_alerts
now tracks <sleeve>.fired per name, diffs day-over-day, and emits a clean
"🧬 New catalyst signal(s)" card on new entrants, tagged Phase-1 paper-validation.
They fire rarely (0 today) → low-noise, high-value. Snapshot re-seeded.

Breakout is already covered by the entry-watcher (✗ unproven tag, same R:R floor).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-06-15.xlsx
+++ b/cache/open_items_2026-06-15.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N296"/>
+  <dimension ref="A1:N297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -12278,13 +12278,13 @@
       </c>
       <c r="N211" s="8" t="inlineStr"/>
     </row>
-    <row r="212" ht="90" customHeight="1">
+    <row r="212" ht="75" customHeight="1">
       <c r="A212" s="2" t="n">
         <v>211</v>
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>WEEKEND-PHANTOMS</t>
+          <t>SLEEVE-ALERTS</t>
         </is>
       </c>
       <c r="C212" s="10" t="inlineStr">
@@ -12294,22 +12294,22 @@
       </c>
       <c r="D212" s="5" t="inlineStr">
         <is>
-          <t>Audit Trail / Data Quality</t>
+          <t>Alerts</t>
         </is>
       </c>
       <c r="E212" s="6" t="inlineStr">
         <is>
-          <t>Weekend pick_dates (Sat/Sun) in audit ledger</t>
+          <t>Dedicated catalyst-sleeve signal alerts</t>
         </is>
       </c>
       <c r="F212" s="5" t="inlineStr">
         <is>
-          <t>signal_log writes pick_date as today.isoformat() — when scan runs on weekend (manual rerun), produces Sat/Sun dates EODHD can't price. 355 such phantoms in ledger. Fix: snap weekend dates forward to next Monday at both write-time (signal_tracker.log_signals) and build-time (build_audit_ledger.py). Preserves original via pick_date_orig field</t>
+          <t>Entry-watcher covers price-action setups (pullback/breakout/impulse) but the 7 catalyst sleeves (PEAD/Insider/ESP/MeanRev/Momentum/DefRot) had no dedicated alert — they only reached Slack indirectly via flip/elite digests. Per principle 14 these are the higher-mechanism signals (PEAD PF 2.04, Momentum 1.53)</t>
         </is>
       </c>
       <c r="G212" s="5" t="inlineStr">
         <is>
-          <t>signal_tracker.py log_signals dow snap + build_audit_ledger.py _compute_returns_for_ticker snap-forward · 353 records normalized · 2 residual edge cases</t>
+          <t>signal_alerts.py: added SLEEVES dimension; _current_state tracks &lt;field&gt;.fired per sleeve; daily diff emits '🧬 New catalyst signal(s)' clean card on new entrants; Phase-1 paper-validation note. Fire rarely (0 today) so low-noise/high-value. Snapshot re-seeded with sleeves key</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr"/>
@@ -12322,23 +12322,23 @@
       </c>
       <c r="L212" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M212" s="3" t="inlineStr">
         <is>
-          <t>e48edac16</t>
+          <t>fa8835903</t>
         </is>
       </c>
       <c r="N212" s="8" t="inlineStr"/>
     </row>
-    <row r="213" ht="75" customHeight="1">
+    <row r="213" ht="90" customHeight="1">
       <c r="A213" s="2" t="n">
         <v>212</v>
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>BT-GUARD-1</t>
+          <t>WEEKEND-PHANTOMS</t>
         </is>
       </c>
       <c r="C213" s="10" t="inlineStr">
@@ -12348,22 +12348,22 @@
       </c>
       <c r="D213" s="5" t="inlineStr">
         <is>
-          <t>Backtest Infrastructure</t>
+          <t>Audit Trail / Data Quality</t>
         </is>
       </c>
       <c r="E213" s="6" t="inlineStr">
         <is>
-          <t>Backtest min_score guard rail</t>
+          <t>Weekend pick_dates (Sat/Sun) in audit ledger</t>
         </is>
       </c>
       <c r="F213" s="5" t="inlineStr">
         <is>
-          <t>Users (and Claude sessions) repeatedly ran 252d backtests with --min-score 65 (live threshold) producing 0 BUYs across all 252 days. Historical scoring is structurally suppressed because sentiment/options/catalyst pillars depend on real-time data not in EODHD backfill.</t>
+          <t>signal_log writes pick_date as today.isoformat() — when scan runs on weekend (manual rerun), produces Sat/Sun dates EODHD can't price. 355 such phantoms in ledger. Fix: snap weekend dates forward to next Monday at both write-time (signal_tracker.log_signals) and build-time (build_audit_ledger.py). Preserves original via pick_date_orig field</t>
         </is>
       </c>
       <c r="G213" s="5" t="inlineStr">
         <is>
-          <t>backtest.py main() now warns loudly when --min-score &gt; 55 (backtest-safe floor). New --accept-low-buys flag silences the warning for legitimate grid-search explorations. --smoke bypasses the guard. Plus diagnostic doc: docs/backtest_historical_scoring_diagnostic.md.</t>
+          <t>signal_tracker.py log_signals dow snap + build_audit_ledger.py _compute_returns_for_ticker snap-forward · 353 records normalized · 2 residual edge cases</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr"/>
@@ -12381,18 +12381,18 @@
       </c>
       <c r="M213" s="3" t="inlineStr">
         <is>
-          <t>d754830</t>
+          <t>e48edac16</t>
         </is>
       </c>
       <c r="N213" s="8" t="inlineStr"/>
     </row>
-    <row r="214" ht="60" customHeight="1">
+    <row r="214" ht="75" customHeight="1">
       <c r="A214" s="2" t="n">
         <v>213</v>
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>LENS-PLAN-PERMODE-TARGETS</t>
+          <t>BT-GUARD-1</t>
         </is>
       </c>
       <c r="C214" s="10" t="inlineStr">
@@ -12402,22 +12402,22 @@
       </c>
       <c r="D214" s="5" t="inlineStr">
         <is>
-          <t>BullVeda · Plan</t>
+          <t>Backtest Infrastructure</t>
         </is>
       </c>
       <c r="E214" s="6" t="inlineStr">
         <is>
-          <t>lens-plan synthesizes per-mode targets by scaling swing levels</t>
+          <t>Backtest min_score guard rail</t>
         </is>
       </c>
       <c r="F214" s="5" t="inlineStr">
         <is>
-          <t>modeAdjust() in lens-plan.jsx scales swing stop/t1/t2 by fixed multipliers (POSITION 0.96/1.10/1.18, INVEST 0.84/1.32/1.58) instead of binding canonical per-mode targets.</t>
+          <t>Users (and Claude sessions) repeatedly ran 252d backtests with --min-score 65 (live threshold) producing 0 BUYs across all 252 days. Historical scoring is structurally suppressed because sentiment/options/catalyst pillars depend on real-time data not in EODHD backfill.</t>
         </is>
       </c>
       <c r="G214" s="5" t="inlineStr">
         <is>
-          <t>Bind per-mode stop/T1/T2/RR from /api/trade_engine?mode= (already fetched by Overview into STATE.payloads). Verdict already fixed to bind decisionsByMode 2026-06-09.</t>
+          <t>backtest.py main() now warns loudly when --min-score &gt; 55 (backtest-safe floor). New --accept-low-buys flag silences the warning for legitimate grid-search explorations. --smoke bypasses the guard. Plus diagnostic doc: docs/backtest_historical_scoring_diagnostic.md.</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr"/>
@@ -12430,23 +12430,23 @@
       </c>
       <c r="L214" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M214" s="3" t="inlineStr">
         <is>
-          <t>99cff7117</t>
+          <t>d754830</t>
         </is>
       </c>
       <c r="N214" s="8" t="inlineStr"/>
     </row>
-    <row r="215" ht="45" customHeight="1">
+    <row r="215" ht="60" customHeight="1">
       <c r="A215" s="2" t="n">
         <v>214</v>
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>SURFACE-WATCHLIST-MOCK</t>
+          <t>LENS-PLAN-PERMODE-TARGETS</t>
         </is>
       </c>
       <c r="C215" s="10" t="inlineStr">
@@ -12456,22 +12456,22 @@
       </c>
       <c r="D215" s="5" t="inlineStr">
         <is>
-          <t>BullVeda · Watchlist</t>
+          <t>BullVeda · Plan</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
         <is>
-          <t>surface-watchlist enrichWL fabricates row data from charCodeAt</t>
+          <t>lens-plan synthesizes per-mode targets by scaling swing levels</t>
         </is>
       </c>
       <c r="F215" s="5" t="inlineStr">
         <is>
-          <t>enrichWL() synthesizes rs/rvol/rr/earn/iv/wlb/n/pf/insider/sent (and conviction tier) from sym char codes — mock, not real data.</t>
+          <t>modeAdjust() in lens-plan.jsx scales swing stop/t1/t2 by fixed multipliers (POSITION 0.96/1.10/1.18, INVEST 0.84/1.32/1.58) instead of binding canonical per-mode targets.</t>
         </is>
       </c>
       <c r="G215" s="5" t="inlineStr">
         <is>
-          <t>Wire enrichWL to the real universe row via BV.scanRow; bind conviction_tier instead of deriving from score.</t>
+          <t>Bind per-mode stop/T1/T2/RR from /api/trade_engine?mode= (already fetched by Overview into STATE.payloads). Verdict already fixed to bind decisionsByMode 2026-06-09.</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr"/>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-1</t>
+          <t>SURFACE-WATCHLIST-MOCK</t>
         </is>
       </c>
       <c r="C216" s="10" t="inlineStr">
@@ -12510,22 +12510,22 @@
       </c>
       <c r="D216" s="5" t="inlineStr">
         <is>
-          <t>Choice C Strategy</t>
+          <t>BullVeda · Watchlist</t>
         </is>
       </c>
       <c r="E216" s="6" t="inlineStr">
         <is>
-          <t>Design doc — docs/strategy_defensive_rotation.md</t>
+          <t>surface-watchlist enrichWL fabricates row data from charCodeAt</t>
         </is>
       </c>
       <c r="F216" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 of Defensive Rotation sleeve build</t>
+          <t>enrichWL() synthesizes rs/rvol/rr/earn/iv/wlb/n/pf/insider/sent (and conviction tier) from sym char codes — mock, not real data.</t>
         </is>
       </c>
       <c r="G216" s="5" t="inlineStr">
         <is>
-          <t>Full design: mechanism, triggers, universe, validation plan</t>
+          <t>Wire enrichWL to the real universe row via BV.scanRow; bind conviction_tier instead of deriving from score.</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr"/>
@@ -12538,12 +12538,12 @@
       </c>
       <c r="L216" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M216" s="3" t="inlineStr">
         <is>
-          <t>399922797</t>
+          <t>99cff7117</t>
         </is>
       </c>
       <c r="N216" s="8" t="inlineStr"/>
@@ -12554,7 +12554,7 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-2</t>
+          <t>DEFROT-1</t>
         </is>
       </c>
       <c r="C217" s="10" t="inlineStr">
@@ -12569,7 +12569,7 @@
       </c>
       <c r="E217" s="6" t="inlineStr">
         <is>
-          <t>Config block — defensive_rotation_sleeve</t>
+          <t>Design doc — docs/strategy_defensive_rotation.md</t>
         </is>
       </c>
       <c r="F217" s="5" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="G217" s="5" t="inlineStr">
         <is>
-          <t>Curated universe, regime gates, sizing, stops; default _enabled=false</t>
+          <t>Full design: mechanism, triggers, universe, validation plan</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr"/>
@@ -12608,7 +12608,7 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-3</t>
+          <t>DEFROT-2</t>
         </is>
       </c>
       <c r="C218" s="10" t="inlineStr">
@@ -12623,7 +12623,7 @@
       </c>
       <c r="E218" s="6" t="inlineStr">
         <is>
-          <t>Detector function — _detect_defensive_rotation</t>
+          <t>Config block — defensive_rotation_sleeve</t>
         </is>
       </c>
       <c r="F218" s="5" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="G218" s="5" t="inlineStr">
         <is>
-          <t>Universe + regime + SPY-50EMA + RS + beta + ATR gates with per-criterion audit</t>
+          <t>Curated universe, regime gates, sizing, stops; default _enabled=false</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr"/>
@@ -12662,7 +12662,7 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-4</t>
+          <t>DEFROT-3</t>
         </is>
       </c>
       <c r="C219" s="10" t="inlineStr">
@@ -12677,7 +12677,7 @@
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>Wire into analyze_ticker</t>
+          <t>Detector function — _detect_defensive_rotation</t>
         </is>
       </c>
       <c r="F219" s="5" t="inlineStr">
@@ -12687,7 +12687,7 @@
       </c>
       <c r="G219" s="5" t="inlineStr">
         <is>
-          <t>Setup family override + trade plan override (1.0 ATR stop, T1+3, T2+6, hold 10-30d, regime exit on SPY 50EMA reclaim)</t>
+          <t>Universe + regime + SPY-50EMA + RS + beta + ATR gates with per-criterion audit</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr"/>
@@ -12716,7 +12716,7 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-5</t>
+          <t>DEFROT-4</t>
         </is>
       </c>
       <c r="C220" s="10" t="inlineStr">
@@ -12731,7 +12731,7 @@
       </c>
       <c r="E220" s="6" t="inlineStr">
         <is>
-          <t>Decision engine bypasses</t>
+          <t>Wire into analyze_ticker</t>
         </is>
       </c>
       <c r="F220" s="5" t="inlineStr">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="G220" s="5" t="inlineStr">
         <is>
-          <t>regime_gate + entry_quality + fund_adequacy bypassed for Defensive Rotation family</t>
+          <t>Setup family override + trade plan override (1.0 ATR stop, T1+3, T2+6, hold 10-30d, regime exit on SPY 50EMA reclaim)</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr"/>
@@ -12770,7 +12770,7 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-6</t>
+          <t>DEFROT-5</t>
         </is>
       </c>
       <c r="C221" s="10" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="E221" s="6" t="inlineStr">
         <is>
-          <t>Universe coverage</t>
+          <t>Decision engine bypasses</t>
         </is>
       </c>
       <c r="F221" s="5" t="inlineStr">
@@ -12795,7 +12795,7 @@
       </c>
       <c r="G221" s="5" t="inlineStr">
         <is>
-          <t>XLP, TLT, IEF added to custom_watchlist (XLU/XLV/GLD already present)</t>
+          <t>regime_gate + entry_quality + fund_adequacy bypassed for Defensive Rotation family</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr"/>
@@ -12824,7 +12824,7 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>DEFROT-7</t>
+          <t>DEFROT-6</t>
         </is>
       </c>
       <c r="C222" s="10" t="inlineStr">
@@ -12839,7 +12839,7 @@
       </c>
       <c r="E222" s="6" t="inlineStr">
         <is>
-          <t>Smoke test + commit</t>
+          <t>Universe coverage</t>
         </is>
       </c>
       <c r="F222" s="5" t="inlineStr">
@@ -12849,7 +12849,7 @@
       </c>
       <c r="G222" s="5" t="inlineStr">
         <is>
-          <t>All 4 detector tests pass; ready for Phase 1 paper validation</t>
+          <t>XLP, TLT, IEF added to custom_watchlist (XLU/XLV/GLD already present)</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr"/>
@@ -12878,7 +12878,7 @@
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-1</t>
+          <t>DEFROT-7</t>
         </is>
       </c>
       <c r="C223" s="10" t="inlineStr">
@@ -12893,17 +12893,17 @@
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion design doc</t>
+          <t>Smoke test + commit</t>
         </is>
       </c>
       <c r="F223" s="5" t="inlineStr">
         <is>
-          <t>Sleeve build</t>
+          <t>Phase 1 of Defensive Rotation sleeve build</t>
         </is>
       </c>
       <c r="G223" s="5" t="inlineStr">
         <is>
-          <t>docs/strategy_mean_reversion.md — full Jegadeesh 1990 mechanism + validation plan</t>
+          <t>All 4 detector tests pass; ready for Phase 1 paper validation</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr"/>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="M223" s="3" t="inlineStr">
         <is>
-          <t>d0c6c4e04</t>
+          <t>399922797</t>
         </is>
       </c>
       <c r="N223" s="8" t="inlineStr"/>
@@ -12932,7 +12932,7 @@
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-2</t>
+          <t>MEANREV-1</t>
         </is>
       </c>
       <c r="C224" s="10" t="inlineStr">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="E224" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion config</t>
+          <t>Mean Reversion design doc</t>
         </is>
       </c>
       <c r="F224" s="5" t="inlineStr">
@@ -12957,7 +12957,7 @@
       </c>
       <c r="G224" s="5" t="inlineStr">
         <is>
-          <t>RSI&lt;30, EMA200 floor, 3-5d hold; default _enabled=true (fires in current choppy regime)</t>
+          <t>docs/strategy_mean_reversion.md — full Jegadeesh 1990 mechanism + validation plan</t>
         </is>
       </c>
       <c r="H224" s="2" t="inlineStr"/>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-3</t>
+          <t>MEANREV-2</t>
         </is>
       </c>
       <c r="C225" s="10" t="inlineStr">
@@ -13001,7 +13001,7 @@
       </c>
       <c r="E225" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion detector</t>
+          <t>Mean Reversion config</t>
         </is>
       </c>
       <c r="F225" s="5" t="inlineStr">
@@ -13011,7 +13011,7 @@
       </c>
       <c r="G225" s="5" t="inlineStr">
         <is>
-          <t>_detect_mean_reversion — 8-gate audit (regime/score/RSI/EMA200/recent_low/RVOL/ADV/earnings)</t>
+          <t>RSI&lt;30, EMA200 floor, 3-5d hold; default _enabled=true (fires in current choppy regime)</t>
         </is>
       </c>
       <c r="H225" s="2" t="inlineStr"/>
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-4</t>
+          <t>MEANREV-3</t>
         </is>
       </c>
       <c r="C226" s="10" t="inlineStr">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="E226" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion wiring</t>
+          <t>Mean Reversion detector</t>
         </is>
       </c>
       <c r="F226" s="5" t="inlineStr">
@@ -13065,7 +13065,7 @@
       </c>
       <c r="G226" s="5" t="inlineStr">
         <is>
-          <t>Setup family override + plan (1.0 ATR stop, +3/+5% T1/T2, 3-5d hold, hard time-stop)</t>
+          <t>_detect_mean_reversion — 8-gate audit (regime/score/RSI/EMA200/recent_low/RVOL/ADV/earnings)</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr"/>
@@ -13094,7 +13094,7 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-5</t>
+          <t>MEANREV-4</t>
         </is>
       </c>
       <c r="C227" s="10" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="E227" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion bypass</t>
+          <t>Mean Reversion wiring</t>
         </is>
       </c>
       <c r="F227" s="5" t="inlineStr">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="G227" s="5" t="inlineStr">
         <is>
-          <t>entry_quality bypass (EXTENDED-down IS the trigger)</t>
+          <t>Setup family override + plan (1.0 ATR stop, +3/+5% T1/T2, 3-5d hold, hard time-stop)</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr"/>
@@ -13148,7 +13148,7 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>MEANREV-6</t>
+          <t>MEANREV-5</t>
         </is>
       </c>
       <c r="C228" s="10" t="inlineStr">
@@ -13163,7 +13163,7 @@
       </c>
       <c r="E228" s="6" t="inlineStr">
         <is>
-          <t>Mean Reversion smoke test</t>
+          <t>Mean Reversion bypass</t>
         </is>
       </c>
       <c r="F228" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="G228" s="5" t="inlineStr">
         <is>
-          <t>4 detector tests pass — fired=True on choppy+RSI=25+EMA200, rejected on RSI=55/below-EMA200/trending</t>
+          <t>entry_quality bypass (EXTENDED-down IS the trigger)</t>
         </is>
       </c>
       <c r="H228" s="2" t="inlineStr"/>
@@ -13202,7 +13202,7 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>PEAD-1</t>
+          <t>MEANREV-6</t>
         </is>
       </c>
       <c r="C229" s="10" t="inlineStr">
@@ -13217,7 +13217,7 @@
       </c>
       <c r="E229" s="6" t="inlineStr">
         <is>
-          <t>PEAD design doc</t>
+          <t>Mean Reversion smoke test</t>
         </is>
       </c>
       <c r="F229" s="5" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="G229" s="5" t="inlineStr">
         <is>
-          <t>docs/strategy_pead.md — Bernard-Thomas 1989, all-regime catalyst sleeve</t>
+          <t>4 detector tests pass — fired=True on choppy+RSI=25+EMA200, rejected on RSI=55/below-EMA200/trending</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr"/>
@@ -13256,7 +13256,7 @@
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>PEAD-2</t>
+          <t>PEAD-1</t>
         </is>
       </c>
       <c r="C230" s="10" t="inlineStr">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="E230" s="6" t="inlineStr">
         <is>
-          <t>PEAD config</t>
+          <t>PEAD design doc</t>
         </is>
       </c>
       <c r="F230" s="5" t="inlineStr">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="G230" s="5" t="inlineStr">
         <is>
-          <t>Day1-3 post-earnings, EPS+5/Rev+2/Gap+3/Revisions&gt;=2, full Kelly with regime caps</t>
+          <t>docs/strategy_pead.md — Bernard-Thomas 1989, all-regime catalyst sleeve</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr"/>
@@ -13310,7 +13310,7 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>PEAD-3</t>
+          <t>PEAD-2</t>
         </is>
       </c>
       <c r="C231" s="10" t="inlineStr">
@@ -13325,7 +13325,7 @@
       </c>
       <c r="E231" s="6" t="inlineStr">
         <is>
-          <t>PEAD detector</t>
+          <t>PEAD config</t>
         </is>
       </c>
       <c r="F231" s="5" t="inlineStr">
@@ -13335,7 +13335,7 @@
       </c>
       <c r="G231" s="5" t="inlineStr">
         <is>
-          <t>_detect_pead — 7-gate audit; regime-independent</t>
+          <t>Day1-3 post-earnings, EPS+5/Rev+2/Gap+3/Revisions&gt;=2, full Kelly with regime caps</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr"/>
@@ -13364,7 +13364,7 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>PEAD-4</t>
+          <t>PEAD-3</t>
         </is>
       </c>
       <c r="C232" s="10" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="E232" s="6" t="inlineStr">
         <is>
-          <t>PEAD wiring</t>
+          <t>PEAD detector</t>
         </is>
       </c>
       <c r="F232" s="5" t="inlineStr">
@@ -13389,7 +13389,7 @@
       </c>
       <c r="G232" s="5" t="inlineStr">
         <is>
-          <t>Setup family override + plan (1.0 ATR stop, +5/+10/+15 targets, 10-30d drift hold)</t>
+          <t>_detect_pead — 7-gate audit; regime-independent</t>
         </is>
       </c>
       <c r="H232" s="2" t="inlineStr"/>
@@ -13418,7 +13418,7 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>PEAD-5</t>
+          <t>PEAD-4</t>
         </is>
       </c>
       <c r="C233" s="10" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>PEAD bypasses</t>
+          <t>PEAD wiring</t>
         </is>
       </c>
       <c r="F233" s="5" t="inlineStr">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G233" s="5" t="inlineStr">
         <is>
-          <t>regime_gate bypassed (catalyst regime-independent), entry_quality bypassed (gap-up IS trigger)</t>
+          <t>Setup family override + plan (1.0 ATR stop, +5/+10/+15 targets, 10-30d drift hold)</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr"/>
@@ -13472,7 +13472,7 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>PEAD-6</t>
+          <t>PEAD-5</t>
         </is>
       </c>
       <c r="C234" s="10" t="inlineStr">
@@ -13487,7 +13487,7 @@
       </c>
       <c r="E234" s="6" t="inlineStr">
         <is>
-          <t>PEAD smoke test</t>
+          <t>PEAD bypasses</t>
         </is>
       </c>
       <c r="F234" s="5" t="inlineStr">
@@ -13497,7 +13497,7 @@
       </c>
       <c r="G234" s="5" t="inlineStr">
         <is>
-          <t>Perfect-setup test fires with all 7 audit checks ✓</t>
+          <t>regime_gate bypassed (catalyst regime-independent), entry_quality bypassed (gap-up IS trigger)</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr"/>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>CLEANUP-HOT-SECTORS</t>
+          <t>PEAD-6</t>
         </is>
       </c>
       <c r="C235" s="10" t="inlineStr">
@@ -13536,22 +13536,22 @@
       </c>
       <c r="D235" s="5" t="inlineStr">
         <is>
-          <t>Code Hygiene / Signal Scanner</t>
+          <t>Choice C Strategy</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
         <is>
-          <t>Remove dead panelHotSectors function</t>
+          <t>PEAD smoke test</t>
         </is>
       </c>
       <c r="F235" s="5" t="inlineStr">
         <is>
-          <t>User asked to remove Hot Sectors panel from grid earlier; function left in file as dead code. Removed 53 lines.</t>
+          <t>Sleeve build</t>
         </is>
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner module · panelHotSectors() deleted</t>
+          <t>Perfect-setup test fires with all 7 audit checks ✓</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr"/>
@@ -13564,23 +13564,23 @@
       </c>
       <c r="L235" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="M235" s="3" t="inlineStr">
         <is>
-          <t>e48edac16</t>
+          <t>d0c6c4e04</t>
         </is>
       </c>
       <c r="N235" s="8" t="inlineStr"/>
     </row>
-    <row r="236" ht="105" customHeight="1">
+    <row r="236" ht="45" customHeight="1">
       <c r="A236" s="2" t="n">
         <v>235</v>
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>UI-CRYPTO-1</t>
+          <t>CLEANUP-HOT-SECTORS</t>
         </is>
       </c>
       <c r="C236" s="10" t="inlineStr">
@@ -13590,22 +13590,22 @@
       </c>
       <c r="D236" s="5" t="inlineStr">
         <is>
-          <t>Crypto Tab</t>
+          <t>Code Hygiene / Signal Scanner</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
         <is>
-          <t>20yr HF analyst Crypto tab rebuild</t>
+          <t>Remove dead panelHotSectors function</t>
         </is>
       </c>
       <c r="F236" s="5" t="inlineStr">
         <is>
-          <t>Crypto tab was stub with 4 cards of placeholder data. Needed a senior HF/Graham-Buffett/swing-trader fused lens for the 24/7 risk-asset bellwether.</t>
+          <t>User asked to remove Hot Sectors panel from grid earlier; function left in file as dead code. Removed 53 lines.</t>
         </is>
       </c>
       <c r="G236" s="5" t="inlineStr">
         <is>
-          <t>13-section renderCrypto in kairos.html: cycle posture banner (Pi-Cycle/MVRV-Z/NUPL/200wk MA), spot KPIs, Graham margin-of-safety floors (realized price, thermo-cap, cost of production, LTH/STH cost), ETH owner-earnings DCF, BTC hard-money compounding, stablecoin liquidity, macro drivers, spot ETF flows, derivatives tape, on-chain valuation composite, catalyst calendar, adjacent equities, L1/L2 rotation, regime-conditional playbook, pre-mortem.</t>
+          <t>kairos.html QuantScanner module · panelHotSectors() deleted</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr"/>
@@ -13623,18 +13623,18 @@
       </c>
       <c r="M236" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
+          <t>e48edac16</t>
         </is>
       </c>
       <c r="N236" s="8" t="inlineStr"/>
     </row>
-    <row r="237" ht="75" customHeight="1">
+    <row r="237" ht="105" customHeight="1">
       <c r="A237" s="2" t="n">
         <v>236</v>
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-T1CAT-1</t>
+          <t>UI-CRYPTO-1</t>
         </is>
       </c>
       <c r="C237" s="10" t="inlineStr">
@@ -13644,22 +13644,22 @@
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Crypto Tab</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
         <is>
-          <t>T1 CATALYST pill read wrong field</t>
+          <t>20yr HF analyst Crypto tab rebuild</t>
         </is>
       </c>
       <c r="F237" s="5" t="inlineStr">
         <is>
-          <t>The scanner '⚡ T1 CATALYST' pill filtered t.tier===T1 (conviction_tier), not the catalyst tier. conviction_tier has 0 T1s on a no-BUY day (CPI blackout: AVOID 928/WATCH 133/T3 14), so the pill matched nothing — while catalyst_tier T1 = 239 names.</t>
+          <t>Crypto tab was stub with 4 cards of placeholder data. Needed a senior HF/Graham-Buffett/swing-trader fused lens for the 24/7 risk-asset bellwether.</t>
         </is>
       </c>
       <c r="G237" s="5" t="inlineStr">
         <is>
-          <t>Changed the pill filter to t.cat===T1 (catalyst tier, matching the displayed CAT column). Rebuilt.</t>
+          <t>13-section renderCrypto in kairos.html: cycle posture banner (Pi-Cycle/MVRV-Z/NUPL/200wk MA), spot KPIs, Graham margin-of-safety floors (realized price, thermo-cap, cost of production, LTH/STH cost), ETH owner-earnings DCF, BTC hard-money compounding, stablecoin liquidity, macro drivers, spot ETF flows, derivatives tape, on-chain valuation composite, catalyst calendar, adjacent equities, L1/L2 rotation, regime-conditional playbook, pre-mortem.</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr"/>
@@ -13672,12 +13672,12 @@
       </c>
       <c r="L237" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M237" s="3" t="inlineStr">
         <is>
-          <t>1d6fdb14a</t>
+          <t>696731a4d</t>
         </is>
       </c>
       <c r="N237" s="8" t="inlineStr"/>
@@ -13688,7 +13688,7 @@
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>EODHD-EDGAR-FUNDAMENTALS</t>
+          <t>SCANNER-T1CAT-1</t>
         </is>
       </c>
       <c r="C238" s="10" t="inlineStr">
@@ -13698,22 +13698,22 @@
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>Data / SEC EDGAR (future quality)</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
         <is>
-          <t>Offload fundamentals to SEC EDGAR (FIX 4)</t>
+          <t>T1 CATALYST pill read wrong field</t>
         </is>
       </c>
       <c r="F238" s="5" t="inlineStr">
         <is>
-          <t>new edgar_client.py behind data_fetcher interface; data.sec.gov companyfacts (User-Agent + &lt;=10 req/s); map XBRL tags to fundamentals.db; nightly batch. Quality upgrade (point-in-time, fixes audit #1/#4) + zeroes per-ticker EODHD fundamentals calls.</t>
+          <t>The scanner '⚡ T1 CATALYST' pill filtered t.tier===T1 (conviction_tier), not the catalyst tier. conviction_tier has 0 T1s on a no-BUY day (CPI blackout: AVOID 928/WATCH 133/T3 14), so the pill matched nothing — while catalyst_tier T1 = 239 names.</t>
         </is>
       </c>
       <c r="G238" s="5" t="inlineStr">
         <is>
-          <t>edgar_client.py + nightly batch</t>
+          <t>Changed the pill filter to t.cat===T1 (catalyst tier, matching the displayed CAT column). Rebuilt.</t>
         </is>
       </c>
       <c r="H238" s="2" t="inlineStr"/>
@@ -13726,12 +13726,12 @@
       </c>
       <c r="L238" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="M238" s="3" t="inlineStr">
         <is>
-          <t>5d05268ef</t>
+          <t>1d6fdb14a</t>
         </is>
       </c>
       <c r="N238" s="8" t="inlineStr"/>
@@ -13742,7 +13742,7 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-QUAL-REASON-1</t>
+          <t>EODHD-EDGAR-FUNDAMENTALS</t>
         </is>
       </c>
       <c r="C239" s="10" t="inlineStr">
@@ -13752,22 +13752,22 @@
       </c>
       <c r="D239" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine</t>
+          <t>Data / SEC EDGAR (future quality)</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
         <is>
-          <t>Misleading entry_quality WATCH reason</t>
+          <t>Offload fundamentals to SEC EDGAR (FIX 4)</t>
         </is>
       </c>
       <c r="F239" s="5" t="inlineStr">
         <is>
-          <t>make_decision hardcoded 'broke through resistance, wait for next base' for ALL MISSED entries — false when stock is below recent high (BFH: MISSED via &gt;2 ATR over EMA21 but 2.1% BELOW 20d high)</t>
+          <t>new edgar_client.py behind data_fetcher interface; data.sec.gov companyfacts (User-Agent + &lt;=10 req/s); map XBRL tags to fundamentals.db; nightly batch. Quality upgrade (point-in-time, fixes audit #1/#4) + zeroes per-ticker EODHD fundamentals calls.</t>
         </is>
       </c>
       <c r="G239" s="5" t="inlineStr">
         <is>
-          <t>classify_entry_quality_detail() returns (label, live-distance reason) naming the actual trigger + honest 'still X% below resistance (not a breakout)' qualifier; threaded entry_quality_reason through make_decision + compute_decisions_by_mode</t>
+          <t>edgar_client.py + nightly batch</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr"/>
@@ -13780,23 +13780,23 @@
       </c>
       <c r="L239" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M239" s="3" t="inlineStr">
         <is>
-          <t>613f10e35</t>
+          <t>5d05268ef</t>
         </is>
       </c>
       <c r="N239" s="8" t="inlineStr"/>
     </row>
-    <row r="240" ht="60" customHeight="1">
+    <row r="240" ht="75" customHeight="1">
       <c r="A240" s="2" t="n">
         <v>239</v>
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>SETDETAIL-FALLBACK</t>
+          <t>ENTRY-QUAL-REASON-1</t>
         </is>
       </c>
       <c r="C240" s="10" t="inlineStr">
@@ -13806,22 +13806,22 @@
       </c>
       <c r="D240" s="5" t="inlineStr">
         <is>
-          <t>Detail UI / Routing</t>
+          <t>Decision Engine</t>
         </is>
       </c>
       <c r="E240" s="6" t="inlineStr">
         <is>
-          <t>setDetailTicker failed for R2000-only tickers</t>
+          <t>Misleading entry_quality WATCH reason</t>
         </is>
       </c>
       <c r="F240" s="5" t="inlineStr">
         <is>
-          <t>Clicking ML Edge picks not in scan bundle (HOOD, ARES, STEM etc.) printed '[kairos] ticker not in scan' and never opened. Now synthesizes minimal t row from window.__mlEdgeCache so detail page opens with _fromMlEdge:true flag</t>
+          <t>make_decision hardcoded 'broke through resistance, wait for next base' for ALL MISSED entries — false when stock is below recent high (BFH: MISSED via &gt;2 ATR over EMA21 but 2.1% BELOW 20d high)</t>
         </is>
       </c>
       <c r="G240" s="5" t="inlineStr">
         <is>
-          <t>kairos.html window.setDetailTicker fallback block</t>
+          <t>classify_entry_quality_detail() returns (label, live-distance reason) naming the actual trigger + honest 'still X% below resistance (not a breakout)' qualifier; threaded entry_quality_reason through make_decision + compute_decisions_by_mode</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr"/>
@@ -13834,12 +13834,12 @@
       </c>
       <c r="L240" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="M240" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
+          <t>613f10e35</t>
         </is>
       </c>
       <c r="N240" s="8" t="inlineStr"/>
@@ -13850,7 +13850,7 @@
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>SETDETAIL-FALLBACK</t>
         </is>
       </c>
       <c r="C241" s="10" t="inlineStr">
@@ -13860,34 +13860,26 @@
       </c>
       <c r="D241" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Detail UI / Routing</t>
         </is>
       </c>
       <c r="E241" s="6" t="inlineStr">
         <is>
-          <t>Update CLAUDE.md with new tools</t>
+          <t>setDetailTicker failed for R2000-only tickers</t>
         </is>
       </c>
       <c r="F241" s="5" t="inlineStr">
         <is>
-          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
+          <t>Clicking ML Edge picks not in scan bundle (HOOD, ARES, STEM etc.) printed '[kairos] ticker not in scan' and never opened. Now synthesizes minimal t row from window.__mlEdgeCache so detail page opens with _fromMlEdge:true flag</t>
         </is>
       </c>
       <c r="G241" s="5" t="inlineStr">
         <is>
-          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
-        </is>
-      </c>
-      <c r="H241" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I241" s="5" t="inlineStr">
-        <is>
-          <t>Win: future Claude sessions discover new tools.</t>
-        </is>
-      </c>
+          <t>kairos.html window.setDetailTicker fallback block</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr"/>
+      <c r="I241" s="5" t="inlineStr"/>
       <c r="J241" s="5" t="inlineStr"/>
       <c r="K241" s="12" t="inlineStr">
         <is>
@@ -13896,27 +13888,23 @@
       </c>
       <c r="L241" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="M241" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N241" s="8" t="inlineStr">
-        <is>
-          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="242" ht="75" customHeight="1">
+          <t>27fd646b1</t>
+        </is>
+      </c>
+      <c r="N241" s="8" t="inlineStr"/>
+    </row>
+    <row r="242" ht="60" customHeight="1">
       <c r="A242" s="2" t="n">
         <v>241</v>
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C242" s="10" t="inlineStr">
@@ -13931,17 +13919,17 @@
       </c>
       <c r="E242" s="6" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
+          <t>Update CLAUDE.md with new tools</t>
         </is>
       </c>
       <c r="F242" s="5" t="inlineStr">
         <is>
-          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
+          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
         </is>
       </c>
       <c r="G242" s="5" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
+          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
         </is>
       </c>
       <c r="H242" s="2" t="inlineStr">
@@ -13951,14 +13939,10 @@
       </c>
       <c r="I242" s="5" t="inlineStr">
         <is>
-          <t>Win: clear activation procedure before flipping live.</t>
-        </is>
-      </c>
-      <c r="J242" s="5" t="inlineStr">
-        <is>
-          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
-        </is>
-      </c>
+          <t>Win: future Claude sessions discover new tools.</t>
+        </is>
+      </c>
+      <c r="J242" s="5" t="inlineStr"/>
       <c r="K242" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13971,12 +13955,12 @@
       </c>
       <c r="M242" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N242" s="8" t="inlineStr">
         <is>
-          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
         </is>
       </c>
     </row>
@@ -13986,7 +13970,7 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>TWO-LOG-DOC</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C243" s="10" t="inlineStr">
@@ -14001,22 +13985,34 @@
       </c>
       <c r="E243" s="6" t="inlineStr">
         <is>
-          <t>Two-log architecture (picks_history vs signal_log) was undocumented</t>
+          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
         </is>
       </c>
       <c r="F243" s="5" t="inlineStr">
         <is>
-          <t>Discovered 2026-05-10 during inflection diagnosis: cache/picks_history.json and data/signal_log.json track different realities (61.2% vs 12.7% recent WR). Tracker feedback reads picks_history; drift alerts read signal_log. Mis-attributing which log feeds which consumer wastes diagnostic time.</t>
+          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
         </is>
       </c>
       <c r="G243" s="5" t="inlineStr">
         <is>
-          <t>Add 'Two-Log Architecture' section to CLAUDE.md after EODHD section, with table mapping consumers + WR snapshots. Cross-reference portfolio_state.json as the ONLY real-trades log.</t>
-        </is>
-      </c>
-      <c r="H243" s="2" t="inlineStr"/>
-      <c r="I243" s="5" t="inlineStr"/>
-      <c r="J243" s="5" t="inlineStr"/>
+          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I243" s="5" t="inlineStr">
+        <is>
+          <t>Win: clear activation procedure before flipping live.</t>
+        </is>
+      </c>
+      <c r="J243" s="5" t="inlineStr">
+        <is>
+          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
+        </is>
+      </c>
       <c r="K243" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14024,23 +14020,27 @@
       </c>
       <c r="L243" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M243" s="3" t="inlineStr">
         <is>
-          <t>8b06e56ae</t>
-        </is>
-      </c>
-      <c r="N243" s="8" t="inlineStr"/>
-    </row>
-    <row r="244" ht="60" customHeight="1">
+          <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N243" s="8" t="inlineStr">
+        <is>
+          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="75" customHeight="1">
       <c r="A244" s="2" t="n">
         <v>243</v>
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>UI-HELP-1</t>
+          <t>TWO-LOG-DOC</t>
         </is>
       </c>
       <c r="C244" s="10" t="inlineStr">
@@ -14050,22 +14050,22 @@
       </c>
       <c r="D244" s="5" t="inlineStr">
         <is>
-          <t>Help System</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E244" s="6" t="inlineStr">
         <is>
-          <t>Help registry expanded 14 to 38 entries</t>
+          <t>Two-log architecture (picks_history vs signal_log) was undocumented</t>
         </is>
       </c>
       <c r="F244" s="5" t="inlineStr">
         <is>
-          <t>Help registry covered only workspace tabs. Detail sub-tabs and MarketsV2 ports had no help content.</t>
+          <t>Discovered 2026-05-10 during inflection diagnosis: cache/picks_history.json and data/signal_log.json track different realities (61.2% vs 12.7% recent WR). Tracker feedback reads picks_history; drift alerts read signal_log. Mis-attributing which log feeds which consumer wastes diagnostic time.</t>
         </is>
       </c>
       <c r="G244" s="5" t="inlineStr">
         <is>
-          <t>Added 24 new entries. kairosHelpFor threads isDetail through dispatcher — prefers detail_ namespace, falls back to bare key. Resolves portfolio workspace vs detail-subtab collision. MarketsV2 render block calls _injectHelpBtn.</t>
+          <t>Add 'Two-Log Architecture' section to CLAUDE.md after EODHD section, with table mapping consumers + WR snapshots. Cross-reference portfolio_state.json as the ONLY real-trades log.</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr"/>
@@ -14078,23 +14078,23 @@
       </c>
       <c r="L244" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M244" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
+          <t>8b06e56ae</t>
         </is>
       </c>
       <c r="N244" s="8" t="inlineStr"/>
     </row>
-    <row r="245" ht="45" customHeight="1">
+    <row r="245" ht="60" customHeight="1">
       <c r="A245" s="2" t="n">
         <v>244</v>
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>UI-HELP-1</t>
         </is>
       </c>
       <c r="C245" s="10" t="inlineStr">
@@ -14104,34 +14104,26 @@
       </c>
       <c r="D245" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Help System</t>
         </is>
       </c>
       <c r="E245" s="6" t="inlineStr">
         <is>
-          <t>Git committer.email set globally</t>
+          <t>Help registry expanded 14 to 38 entries</t>
         </is>
       </c>
       <c r="F245" s="5" t="inlineStr">
         <is>
-          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
+          <t>Help registry covered only workspace tabs. Detail sub-tabs and MarketsV2 ports had no help content.</t>
         </is>
       </c>
       <c r="G245" s="5" t="inlineStr">
         <is>
-          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
-        </is>
-      </c>
-      <c r="H245" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I245" s="5" t="inlineStr">
-        <is>
-          <t>Win: clean attribution in git log.</t>
-        </is>
-      </c>
+          <t>Added 24 new entries. kairosHelpFor threads isDetail through dispatcher — prefers detail_ namespace, falls back to bare key. Resolves portfolio workspace vs detail-subtab collision. MarketsV2 render block calls _injectHelpBtn.</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr"/>
+      <c r="I245" s="5" t="inlineStr"/>
       <c r="J245" s="5" t="inlineStr"/>
       <c r="K245" s="12" t="inlineStr">
         <is>
@@ -14140,27 +14132,23 @@
       </c>
       <c r="L245" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M245" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
-        </is>
-      </c>
-      <c r="N245" s="8" t="inlineStr">
-        <is>
-          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
-        </is>
-      </c>
-    </row>
-    <row r="246" ht="90" customHeight="1">
+          <t>696731a4d</t>
+        </is>
+      </c>
+      <c r="N245" s="8" t="inlineStr"/>
+    </row>
+    <row r="246" ht="45" customHeight="1">
       <c r="A246" s="2" t="n">
         <v>245</v>
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>UI-MLEDGE-1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="C246" s="10" t="inlineStr">
@@ -14170,26 +14158,34 @@
       </c>
       <c r="D246" s="5" t="inlineStr">
         <is>
-          <t>ML Edge Tab</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E246" s="6" t="inlineStr">
         <is>
-          <t>Theme switching + tf-* visual port</t>
+          <t>Git committer.email set globally</t>
         </is>
       </c>
       <c r="F246" s="5" t="inlineStr">
         <is>
-          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
+          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
         </is>
       </c>
       <c r="G246" s="5" t="inlineStr">
         <is>
-          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
-        </is>
-      </c>
-      <c r="H246" s="2" t="inlineStr"/>
-      <c r="I246" s="5" t="inlineStr"/>
+          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I246" s="5" t="inlineStr">
+        <is>
+          <t>Win: clean attribution in git log.</t>
+        </is>
+      </c>
       <c r="J246" s="5" t="inlineStr"/>
       <c r="K246" s="12" t="inlineStr">
         <is>
@@ -14198,23 +14194,27 @@
       </c>
       <c r="L246" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M246" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
-        </is>
-      </c>
-      <c r="N246" s="8" t="inlineStr"/>
-    </row>
-    <row r="247" ht="45" customHeight="1">
+          <t>4129e5565</t>
+        </is>
+      </c>
+      <c r="N246" s="8" t="inlineStr">
+        <is>
+          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="90" customHeight="1">
       <c r="A247" s="2" t="n">
         <v>246</v>
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>IPAD-2</t>
+          <t>UI-MLEDGE-1</t>
         </is>
       </c>
       <c r="C247" s="10" t="inlineStr">
@@ -14224,39 +14224,27 @@
       </c>
       <c r="D247" s="5" t="inlineStr">
         <is>
-          <t>Mobile / iPad</t>
+          <t>ML Edge Tab</t>
         </is>
       </c>
       <c r="E247" s="6" t="inlineStr">
         <is>
-          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
+          <t>Theme switching + tf-* visual port</t>
         </is>
       </c>
       <c r="F247" s="5" t="inlineStr">
         <is>
-          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
+          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
         </is>
       </c>
       <c r="G247" s="5" t="inlineStr">
         <is>
-          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
-        </is>
-      </c>
-      <c r="H247" s="2" t="inlineStr">
-        <is>
-          <t>15 min</t>
-        </is>
-      </c>
-      <c r="I247" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J247" s="5" t="inlineStr">
-        <is>
-          <t>Sub-task of IPAD-1.</t>
-        </is>
-      </c>
+          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr"/>
+      <c r="I247" s="5" t="inlineStr"/>
+      <c r="J247" s="5" t="inlineStr"/>
       <c r="K247" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14264,19 +14252,15 @@
       </c>
       <c r="L247" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M247" s="3" t="inlineStr">
         <is>
-          <t>79fa01a75</t>
-        </is>
-      </c>
-      <c r="N247" s="8" t="inlineStr">
-        <is>
-          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
-        </is>
-      </c>
+          <t>696731a4d</t>
+        </is>
+      </c>
+      <c r="N247" s="8" t="inlineStr"/>
     </row>
     <row r="248" ht="45" customHeight="1">
       <c r="A248" s="2" t="n">
@@ -14284,7 +14268,7 @@
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>SLACK-NEWSLETTER-MLALERT</t>
+          <t>IPAD-2</t>
         </is>
       </c>
       <c r="C248" s="10" t="inlineStr">
@@ -14294,27 +14278,39 @@
       </c>
       <c r="D248" s="5" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile / iPad</t>
         </is>
       </c>
       <c r="E248" s="6" t="inlineStr">
         <is>
-          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
+          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
         </is>
       </c>
       <c r="F248" s="5" t="inlineStr">
         <is>
-          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
+          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
         </is>
       </c>
       <c r="G248" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd + scripts/ml_alert_slack.py</t>
-        </is>
-      </c>
-      <c r="H248" s="2" t="inlineStr"/>
-      <c r="I248" s="5" t="inlineStr"/>
-      <c r="J248" s="5" t="inlineStr"/>
+          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="I248" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J248" s="5" t="inlineStr">
+        <is>
+          <t>Sub-task of IPAD-1.</t>
+        </is>
+      </c>
       <c r="K248" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14322,15 +14318,19 @@
       </c>
       <c r="L248" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M248" s="3" t="inlineStr">
         <is>
-          <t>d1ea97913</t>
-        </is>
-      </c>
-      <c r="N248" s="8" t="inlineStr"/>
+          <t>79fa01a75</t>
+        </is>
+      </c>
+      <c r="N248" s="8" t="inlineStr">
+        <is>
+          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
+        </is>
+      </c>
     </row>
     <row r="249" ht="45" customHeight="1">
       <c r="A249" s="2" t="n">
@@ -14338,7 +14338,7 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>FORENSICS-WEEKLY-SLACK</t>
+          <t>SLACK-NEWSLETTER-MLALERT</t>
         </is>
       </c>
       <c r="C249" s="10" t="inlineStr">
@@ -14348,22 +14348,22 @@
       </c>
       <c r="D249" s="5" t="inlineStr">
         <is>
-          <t>Notifications / Audit</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E249" s="6" t="inlineStr">
         <is>
-          <t>Weekly pick-forensics Slack digest</t>
+          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
         </is>
       </c>
       <c r="F249" s="5" t="inlineStr">
         <is>
-          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
+          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
         </is>
       </c>
       <c r="G249" s="5" t="inlineStr">
         <is>
-          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+          <t>infra/launchd + scripts/ml_alert_slack.py</t>
         </is>
       </c>
       <c r="H249" s="2" t="inlineStr"/>
@@ -14381,18 +14381,18 @@
       </c>
       <c r="M249" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d1ea97913</t>
         </is>
       </c>
       <c r="N249" s="8" t="inlineStr"/>
     </row>
-    <row r="250" ht="75" customHeight="1">
+    <row r="250" ht="45" customHeight="1">
       <c r="A250" s="2" t="n">
         <v>249</v>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
+          <t>FORENSICS-WEEKLY-SLACK</t>
         </is>
       </c>
       <c r="C250" s="10" t="inlineStr">
@@ -14402,39 +14402,27 @@
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Notifications / Audit</t>
         </is>
       </c>
       <c r="E250" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Weekly pick-forensics Slack digest</t>
         </is>
       </c>
       <c r="F250" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
         </is>
       </c>
       <c r="G250" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
-        </is>
-      </c>
-      <c r="H250" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I250" s="5" t="inlineStr">
-        <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
-        </is>
-      </c>
-      <c r="J250" s="5" t="inlineStr">
-        <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
-        </is>
-      </c>
+          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr"/>
+      <c r="I250" s="5" t="inlineStr"/>
+      <c r="J250" s="5" t="inlineStr"/>
       <c r="K250" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14442,27 +14430,23 @@
       </c>
       <c r="L250" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M250" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N250" s="8" t="inlineStr">
-        <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="251" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N250" s="8" t="inlineStr"/>
+    </row>
+    <row r="251" ht="75" customHeight="1">
       <c r="A251" s="2" t="n">
         <v>250</v>
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C251" s="10" t="inlineStr">
@@ -14472,37 +14456,37 @@
       </c>
       <c r="D251" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F251" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G251" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I251" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J251" s="5" t="inlineStr">
         <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K251" s="12" t="inlineStr">
@@ -14512,17 +14496,17 @@
       </c>
       <c r="L251" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M251" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N251" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
         </is>
       </c>
     </row>
@@ -14532,7 +14516,7 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C252" s="10" t="inlineStr">
@@ -14547,32 +14531,32 @@
       </c>
       <c r="E252" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F252" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G252" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I252" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J252" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K252" s="12" t="inlineStr">
@@ -14592,7 +14576,7 @@
       </c>
       <c r="N252" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -14602,7 +14586,7 @@
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C253" s="10" t="inlineStr">
@@ -14617,32 +14601,32 @@
       </c>
       <c r="E253" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F253" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G253" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I253" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J253" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K253" s="12" t="inlineStr">
@@ -14662,7 +14646,7 @@
       </c>
       <c r="N253" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
         </is>
       </c>
     </row>
@@ -14672,7 +14656,7 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>OPS-4</t>
         </is>
       </c>
       <c r="C254" s="10" t="inlineStr">
@@ -14687,32 +14671,32 @@
       </c>
       <c r="E254" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F254" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G254" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I254" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J254" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K254" s="12" t="inlineStr">
@@ -14722,27 +14706,27 @@
       </c>
       <c r="L254" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M254" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N254" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="255" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="60" customHeight="1">
       <c r="A255" s="2" t="n">
         <v>254</v>
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>SCAN-FAILURE-ALERT</t>
+          <t>OPS-5</t>
         </is>
       </c>
       <c r="C255" s="10" t="inlineStr">
@@ -14752,27 +14736,39 @@
       </c>
       <c r="D255" s="5" t="inlineStr">
         <is>
-          <t>Ops / Alerts</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
         <is>
-          <t>Scan-failure + EODHD-quota Slack alert</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F255" s="5" t="inlineStr">
         <is>
-          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G255" s="5" t="inlineStr">
         <is>
-          <t>swing_trade.py exit hook</t>
-        </is>
-      </c>
-      <c r="H255" s="2" t="inlineStr"/>
-      <c r="I255" s="5" t="inlineStr"/>
-      <c r="J255" s="5" t="inlineStr"/>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I255" s="5" t="inlineStr">
+        <is>
+          <t>Win: fast iteration on report templates.</t>
+        </is>
+      </c>
+      <c r="J255" s="5" t="inlineStr">
+        <is>
+          <t>Trivial CLI wrapper.</t>
+        </is>
+      </c>
       <c r="K255" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14780,15 +14776,19 @@
       </c>
       <c r="L255" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M255" s="3" t="inlineStr">
         <is>
-          <t>0dc7675ee</t>
-        </is>
-      </c>
-      <c r="N255" s="8" t="inlineStr"/>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N255" s="8" t="inlineStr">
+        <is>
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="45" customHeight="1">
       <c r="A256" s="2" t="n">
@@ -14796,7 +14796,7 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
+          <t>SCAN-FAILURE-ALERT</t>
         </is>
       </c>
       <c r="C256" s="10" t="inlineStr">
@@ -14806,22 +14806,22 @@
       </c>
       <c r="D256" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Alerts</t>
         </is>
       </c>
       <c r="E256" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot: load or retire</t>
+          <t>Scan-failure + EODHD-quota Slack alert</t>
         </is>
       </c>
       <c r="F256" s="5" t="inlineStr">
         <is>
-          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
+          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
         </is>
       </c>
       <c r="G256" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd</t>
+          <t>swing_trade.py exit hook</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr"/>
@@ -14844,13 +14844,13 @@
       </c>
       <c r="N256" s="8" t="inlineStr"/>
     </row>
-    <row r="257" ht="60" customHeight="1">
+    <row r="257" ht="45" customHeight="1">
       <c r="A257" s="2" t="n">
         <v>256</v>
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>OVERVIEW-TQ-LABEL</t>
+          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
         </is>
       </c>
       <c r="C257" s="10" t="inlineStr">
@@ -14860,22 +14860,22 @@
       </c>
       <c r="D257" s="5" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
         <is>
-          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
+          <t>Decide momentum-snapshot: load or retire</t>
         </is>
       </c>
       <c r="F257" s="5" t="inlineStr">
         <is>
-          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
+          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
         </is>
       </c>
       <c r="G257" s="5" t="inlineStr">
         <is>
-          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
+          <t>infra/launchd</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr"/>
@@ -14888,23 +14888,23 @@
       </c>
       <c r="L257" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M257" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>0dc7675ee</t>
         </is>
       </c>
       <c r="N257" s="8" t="inlineStr"/>
     </row>
-    <row r="258" ht="150" customHeight="1">
+    <row r="258" ht="60" customHeight="1">
       <c r="A258" s="2" t="n">
         <v>257</v>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>OVERVIEW-TQ-LABEL</t>
         </is>
       </c>
       <c r="C258" s="10" t="inlineStr">
@@ -14914,31 +14914,27 @@
       </c>
       <c r="D258" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="E258" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
         </is>
       </c>
       <c r="F258" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
         </is>
       </c>
       <c r="G258" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr"/>
       <c r="I258" s="5" t="inlineStr"/>
-      <c r="J258" s="5" t="inlineStr">
-        <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
-        </is>
-      </c>
+      <c r="J258" s="5" t="inlineStr"/>
       <c r="K258" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -14946,27 +14942,23 @@
       </c>
       <c r="L258" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M258" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
-        </is>
-      </c>
-      <c r="N258" s="8" t="inlineStr">
-        <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="259" ht="105" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N258" s="8" t="inlineStr"/>
+    </row>
+    <row r="259" ht="150" customHeight="1">
       <c r="A259" s="2" t="n">
         <v>258</v>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>SMC-OB-DISPLAY-1</t>
+          <t>PERF-7b</t>
         </is>
       </c>
       <c r="C259" s="10" t="inlineStr">
@@ -14976,27 +14968,31 @@
       </c>
       <c r="D259" s="5" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E259" s="6" t="inlineStr">
         <is>
-          <t>OB confluence badges in SMC tab</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F259" s="5" t="inlineStr">
         <is>
-          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G259" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr"/>
       <c r="I259" s="5" t="inlineStr"/>
-      <c r="J259" s="5" t="inlineStr"/>
+      <c r="J259" s="5" t="inlineStr">
+        <is>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+        </is>
+      </c>
       <c r="K259" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15004,23 +15000,27 @@
       </c>
       <c r="L259" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M259" s="3" t="inlineStr">
         <is>
-          <t>8182c3977</t>
-        </is>
-      </c>
-      <c r="N259" s="8" t="inlineStr"/>
-    </row>
-    <row r="260" ht="45" customHeight="1">
+          <t>cf30df858</t>
+        </is>
+      </c>
+      <c r="N259" s="8" t="inlineStr">
+        <is>
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="105" customHeight="1">
       <c r="A260" s="2" t="n">
         <v>259</v>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-1</t>
+          <t>SMC-OB-DISPLAY-1</t>
         </is>
       </c>
       <c r="C260" s="10" t="inlineStr">
@@ -15030,22 +15030,22 @@
       </c>
       <c r="D260" s="5" t="inlineStr">
         <is>
-          <t>Sharpe Roadmap</t>
+          <t>SMC</t>
         </is>
       </c>
       <c r="E260" s="6" t="inlineStr">
         <is>
-          <t>Sharpe gate in momentum detector</t>
+          <t>OB confluence badges in SMC tab</t>
         </is>
       </c>
       <c r="F260" s="5" t="inlineStr">
         <is>
-          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
+          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
         </is>
       </c>
       <c r="G260" s="5" t="inlineStr">
         <is>
-          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
+          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr"/>
@@ -15058,12 +15058,12 @@
       </c>
       <c r="L260" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="M260" s="3" t="inlineStr">
         <is>
-          <t>dbbd6b5f6</t>
+          <t>8182c3977</t>
         </is>
       </c>
       <c r="N260" s="8" t="inlineStr"/>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-10</t>
+          <t>SHARPE-1</t>
         </is>
       </c>
       <c r="C261" s="10" t="inlineStr">
@@ -15089,17 +15089,17 @@
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>Sharpe alerts for watchlist</t>
+          <t>Sharpe gate in momentum detector</t>
         </is>
       </c>
       <c r="F261" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
         </is>
       </c>
       <c r="G261" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
+          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr"/>
@@ -15128,7 +15128,7 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-11</t>
+          <t>SHARPE-10</t>
         </is>
       </c>
       <c r="C262" s="10" t="inlineStr">
@@ -15143,17 +15143,17 @@
       </c>
       <c r="E262" s="6" t="inlineStr">
         <is>
-          <t>Per-trade Sharpe attribution</t>
+          <t>Sharpe alerts for watchlist</t>
         </is>
       </c>
       <c r="F262" s="5" t="inlineStr">
         <is>
-          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G262" s="5" t="inlineStr">
         <is>
-          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
+          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr"/>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-12</t>
+          <t>SHARPE-11</t>
         </is>
       </c>
       <c r="C263" s="10" t="inlineStr">
@@ -15197,17 +15197,17 @@
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>Sharpe consistency check</t>
+          <t>Per-trade Sharpe attribution</t>
         </is>
       </c>
       <c r="F263" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
         </is>
       </c>
       <c r="G263" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
+          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr"/>
@@ -15236,7 +15236,7 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-2</t>
+          <t>SHARPE-12</t>
         </is>
       </c>
       <c r="C264" s="10" t="inlineStr">
@@ -15251,17 +15251,17 @@
       </c>
       <c r="E264" s="6" t="inlineStr">
         <is>
-          <t>Sharpe column in v2 dashboard</t>
+          <t>Sharpe consistency check</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
         <is>
-          <t>Surface 126d Sharpe per ticker as sortable column</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G264" s="5" t="inlineStr">
         <is>
-          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
+          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr"/>
@@ -15290,7 +15290,7 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-3</t>
+          <t>SHARPE-2</t>
         </is>
       </c>
       <c r="C265" s="10" t="inlineStr">
@@ -15305,17 +15305,17 @@
       </c>
       <c r="E265" s="6" t="inlineStr">
         <is>
-          <t>Per-stock Sharpe by regime</t>
+          <t>Sharpe column in v2 dashboard</t>
         </is>
       </c>
       <c r="F265" s="5" t="inlineStr">
         <is>
-          <t>Decompose per-stock Sharpe by historical regime tags</t>
+          <t>Surface 126d Sharpe per ticker as sortable column</t>
         </is>
       </c>
       <c r="G265" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
+          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr"/>
@@ -15344,7 +15344,7 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-4</t>
+          <t>SHARPE-3</t>
         </is>
       </c>
       <c r="C266" s="10" t="inlineStr">
@@ -15359,17 +15359,17 @@
       </c>
       <c r="E266" s="6" t="inlineStr">
         <is>
-          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
+          <t>Per-stock Sharpe by regime</t>
         </is>
       </c>
       <c r="F266" s="5" t="inlineStr">
         <is>
-          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
+          <t>Decompose per-stock Sharpe by historical regime tags</t>
         </is>
       </c>
       <c r="G266" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
+          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr"/>
@@ -15398,7 +15398,7 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-5</t>
+          <t>SHARPE-4</t>
         </is>
       </c>
       <c r="C267" s="10" t="inlineStr">
@@ -15413,17 +15413,17 @@
       </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-weighted position sizing</t>
+          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
         </is>
       </c>
       <c r="F267" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
         </is>
       </c>
       <c r="G267" s="5" t="inlineStr">
         <is>
-          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr"/>
@@ -15452,7 +15452,7 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-6</t>
+          <t>SHARPE-5</t>
         </is>
       </c>
       <c r="C268" s="10" t="inlineStr">
@@ -15467,17 +15467,17 @@
       </c>
       <c r="E268" s="6" t="inlineStr">
         <is>
-          <t>Portfolio Sharpe KPI vs target</t>
+          <t>Sharpe-weighted position sizing</t>
         </is>
       </c>
       <c r="F268" s="5" t="inlineStr">
         <is>
-          <t>Annualized Sharpe target tracking + gap report</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G268" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
+          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr"/>
@@ -15506,7 +15506,7 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-7</t>
+          <t>SHARPE-6</t>
         </is>
       </c>
       <c r="C269" s="10" t="inlineStr">
@@ -15521,17 +15521,17 @@
       </c>
       <c r="E269" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-based stop sizing</t>
+          <t>Portfolio Sharpe KPI vs target</t>
         </is>
       </c>
       <c r="F269" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Annualized Sharpe target tracking + gap report</t>
         </is>
       </c>
       <c r="G269" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
         </is>
       </c>
       <c r="H269" s="2" t="inlineStr"/>
@@ -15560,7 +15560,7 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-8</t>
+          <t>SHARPE-7</t>
         </is>
       </c>
       <c r="C270" s="10" t="inlineStr">
@@ -15575,17 +15575,17 @@
       </c>
       <c r="E270" s="6" t="inlineStr">
         <is>
-          <t>Sortino computation alongside Sharpe</t>
+          <t>Sharpe-based stop sizing</t>
         </is>
       </c>
       <c r="F270" s="5" t="inlineStr">
         <is>
-          <t>Downside-only vol denominator added everywhere</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
+          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr"/>
@@ -15614,7 +15614,7 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-9</t>
+          <t>SHARPE-8</t>
         </is>
       </c>
       <c r="C271" s="10" t="inlineStr">
@@ -15629,17 +15629,17 @@
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>SPY-Sharpe regime cross-validation</t>
+          <t>Sortino computation alongside Sharpe</t>
         </is>
       </c>
       <c r="F271" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Downside-only vol denominator added everywhere</t>
         </is>
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
+          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr"/>
@@ -15662,13 +15662,13 @@
       </c>
       <c r="N271" s="8" t="inlineStr"/>
     </row>
-    <row r="272" ht="60" customHeight="1">
+    <row r="272" ht="45" customHeight="1">
       <c r="A272" s="2" t="n">
         <v>271</v>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-RECUR-CHIP</t>
+          <t>SHARPE-9</t>
         </is>
       </c>
       <c r="C272" s="10" t="inlineStr">
@@ -15678,22 +15678,22 @@
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>Signal Scanner</t>
+          <t>Sharpe Roadmap</t>
         </is>
       </c>
       <c r="E272" s="6" t="inlineStr">
         <is>
-          <t>Recurrence chip</t>
+          <t>SPY-Sharpe regime cross-validation</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G272" s="5" t="inlineStr">
         <is>
-          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr"/>
@@ -15706,23 +15706,23 @@
       </c>
       <c r="L272" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M272" s="3" t="inlineStr">
         <is>
-          <t>cf702f2b4</t>
+          <t>dbbd6b5f6</t>
         </is>
       </c>
       <c r="N272" s="8" t="inlineStr"/>
     </row>
-    <row r="273" ht="120" customHeight="1">
+    <row r="273" ht="60" customHeight="1">
       <c r="A273" s="2" t="n">
         <v>272</v>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>CONVICTION-TIER-WIRE</t>
+          <t>SCANNER-RECUR-CHIP</t>
         </is>
       </c>
       <c r="C273" s="10" t="inlineStr">
@@ -15732,39 +15732,27 @@
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Conviction</t>
+          <t>Signal Scanner</t>
         </is>
       </c>
       <c r="E273" s="6" t="inlineStr">
         <is>
-          <t>Conviction tier: simplified to score-band only</t>
+          <t>Recurrence chip</t>
         </is>
       </c>
       <c r="F273" s="5" t="inlineStr">
         <is>
-          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
+          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
         </is>
       </c>
       <c r="G273" s="5" t="inlineStr">
         <is>
-          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
-        </is>
-      </c>
-      <c r="H273" s="2" t="inlineStr">
-        <is>
-          <t>2-4 hrs + backtest validation</t>
-        </is>
-      </c>
-      <c r="I273" s="5" t="inlineStr">
-        <is>
-          <t>Medium — changes live size or eliminates a layer</t>
-        </is>
-      </c>
-      <c r="J273" s="5" t="inlineStr">
-        <is>
-          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
-        </is>
-      </c>
+          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr"/>
+      <c r="I273" s="5" t="inlineStr"/>
+      <c r="J273" s="5" t="inlineStr"/>
       <c r="K273" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15772,27 +15760,23 @@
       </c>
       <c r="L273" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N273" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
-        </is>
-      </c>
-    </row>
-    <row r="274" ht="75" customHeight="1">
+          <t>cf702f2b4</t>
+        </is>
+      </c>
+      <c r="N273" s="8" t="inlineStr"/>
+    </row>
+    <row r="274" ht="120" customHeight="1">
       <c r="A274" s="2" t="n">
         <v>273</v>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-Q-AB</t>
+          <t>CONVICTION-TIER-WIRE</t>
         </is>
       </c>
       <c r="C274" s="10" t="inlineStr">
@@ -15802,27 +15786,39 @@
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Gates</t>
+          <t>Strategy / Conviction</t>
         </is>
       </c>
       <c r="E274" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional entry_quality A/B</t>
+          <t>Conviction tier: simplified to score-band only</t>
         </is>
       </c>
       <c r="F274" s="5" t="inlineStr">
         <is>
-          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
+          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
         </is>
       </c>
       <c r="G274" s="5" t="inlineStr">
         <is>
-          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
-        </is>
-      </c>
-      <c r="H274" s="2" t="inlineStr"/>
-      <c r="I274" s="5" t="inlineStr"/>
-      <c r="J274" s="5" t="inlineStr"/>
+          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>2-4 hrs + backtest validation</t>
+        </is>
+      </c>
+      <c r="I274" s="5" t="inlineStr">
+        <is>
+          <t>Medium — changes live size or eliminates a layer</t>
+        </is>
+      </c>
+      <c r="J274" s="5" t="inlineStr">
+        <is>
+          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
+        </is>
+      </c>
       <c r="K274" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15830,23 +15826,27 @@
       </c>
       <c r="L274" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr">
         <is>
-          <t>07c3af6a3</t>
-        </is>
-      </c>
-      <c r="N274" s="8" t="inlineStr"/>
-    </row>
-    <row r="275" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N274" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="75" customHeight="1">
       <c r="A275" s="2" t="n">
         <v>274</v>
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-1</t>
+          <t>ENTRY-Q-AB</t>
         </is>
       </c>
       <c r="C275" s="10" t="inlineStr">
@@ -15856,22 +15856,22 @@
       </c>
       <c r="D275" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Options Paper</t>
+          <t>Strategy / Gates</t>
         </is>
       </c>
       <c r="E275" s="6" t="inlineStr">
         <is>
-          <t>Signal -&gt; options-structure mapper</t>
+          <t>Regime-conditional entry_quality A/B</t>
         </is>
       </c>
       <c r="F275" s="5" t="inlineStr">
         <is>
-          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
+          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
         </is>
       </c>
       <c r="G275" s="5" t="inlineStr">
         <is>
-          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
+          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr"/>
@@ -15884,23 +15884,23 @@
       </c>
       <c r="L275" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr">
         <is>
-          <t>9c3a2a58d</t>
+          <t>07c3af6a3</t>
         </is>
       </c>
       <c r="N275" s="8" t="inlineStr"/>
     </row>
-    <row r="276" ht="45" customHeight="1">
+    <row r="276" ht="60" customHeight="1">
       <c r="A276" s="2" t="n">
         <v>275</v>
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-2</t>
+          <t>OPT-PAPER-1</t>
         </is>
       </c>
       <c r="C276" s="10" t="inlineStr">
@@ -15915,17 +15915,17 @@
       </c>
       <c r="E276" s="6" t="inlineStr">
         <is>
-          <t>Contract selection from Schwab chain</t>
+          <t>Signal -&gt; options-structure mapper</t>
         </is>
       </c>
       <c r="F276" s="5" t="inlineStr">
         <is>
-          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
+          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
         </is>
       </c>
       <c r="G276" s="5" t="inlineStr">
         <is>
-          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
+          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr"/>
@@ -15948,13 +15948,13 @@
       </c>
       <c r="N276" s="8" t="inlineStr"/>
     </row>
-    <row r="277" ht="60" customHeight="1">
+    <row r="277" ht="45" customHeight="1">
       <c r="A277" s="2" t="n">
         <v>276</v>
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-3</t>
+          <t>OPT-PAPER-2</t>
         </is>
       </c>
       <c r="C277" s="10" t="inlineStr">
@@ -15969,17 +15969,17 @@
       </c>
       <c r="E277" s="6" t="inlineStr">
         <is>
-          <t>Alpaca paper options orders in executor.py</t>
+          <t>Contract selection from Schwab chain</t>
         </is>
       </c>
       <c r="F277" s="5" t="inlineStr">
         <is>
-          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
+          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
         </is>
       </c>
       <c r="G277" s="5" t="inlineStr">
         <is>
-          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
+          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr"/>
@@ -16002,13 +16002,13 @@
       </c>
       <c r="N277" s="8" t="inlineStr"/>
     </row>
-    <row r="278" ht="45" customHeight="1">
+    <row r="278" ht="60" customHeight="1">
       <c r="A278" s="2" t="n">
         <v>277</v>
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-4</t>
+          <t>OPT-PAPER-3</t>
         </is>
       </c>
       <c r="C278" s="10" t="inlineStr">
@@ -16023,17 +16023,17 @@
       </c>
       <c r="E278" s="6" t="inlineStr">
         <is>
-          <t>Options position tracking + contract P&amp;L</t>
+          <t>Alpaca paper options orders in executor.py</t>
         </is>
       </c>
       <c r="F278" s="5" t="inlineStr">
         <is>
-          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
+          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
         </is>
       </c>
       <c r="G278" s="5" t="inlineStr">
         <is>
-          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
+          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr"/>
@@ -16051,7 +16051,7 @@
       </c>
       <c r="M278" s="3" t="inlineStr">
         <is>
-          <t>635ae960f</t>
+          <t>9c3a2a58d</t>
         </is>
       </c>
       <c r="N278" s="8" t="inlineStr"/>
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-5</t>
+          <t>OPT-PAPER-4</t>
         </is>
       </c>
       <c r="C279" s="10" t="inlineStr">
@@ -16077,17 +16077,17 @@
       </c>
       <c r="E279" s="6" t="inlineStr">
         <is>
-          <t>Options-specific exits</t>
+          <t>Options position tracking + contract P&amp;L</t>
         </is>
       </c>
       <c r="F279" s="5" t="inlineStr">
         <is>
-          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
+          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
         </is>
       </c>
       <c r="G279" s="5" t="inlineStr">
         <is>
-          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
+          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr"/>
@@ -16110,13 +16110,13 @@
       </c>
       <c r="N279" s="8" t="inlineStr"/>
     </row>
-    <row r="280" ht="120" customHeight="1">
+    <row r="280" ht="45" customHeight="1">
       <c r="A280" s="2" t="n">
         <v>279</v>
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>UI-STRAT-1</t>
+          <t>OPT-PAPER-5</t>
         </is>
       </c>
       <c r="C280" s="10" t="inlineStr">
@@ -16126,22 +16126,22 @@
       </c>
       <c r="D280" s="5" t="inlineStr">
         <is>
-          <t>Strategy Lab</t>
+          <t>Strategy / Options Paper</t>
         </is>
       </c>
       <c r="E280" s="6" t="inlineStr">
         <is>
-          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
+          <t>Options-specific exits</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
+          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
         </is>
       </c>
       <c r="G280" s="5" t="inlineStr">
         <is>
-          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
+          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr"/>
@@ -16154,23 +16154,23 @@
       </c>
       <c r="L280" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="M280" s="3" t="inlineStr">
         <is>
-          <t>93ec11842</t>
+          <t>635ae960f</t>
         </is>
       </c>
       <c r="N280" s="8" t="inlineStr"/>
     </row>
-    <row r="281" ht="60" customHeight="1">
+    <row r="281" ht="120" customHeight="1">
       <c r="A281" s="2" t="n">
         <v>280</v>
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>TE-STRATEGY-MODE</t>
+          <t>UI-STRAT-1</t>
         </is>
       </c>
       <c r="C281" s="10" t="inlineStr">
@@ -16180,22 +16180,22 @@
       </c>
       <c r="D281" s="5" t="inlineStr">
         <is>
-          <t>Target Engine</t>
+          <t>Strategy Lab</t>
         </is>
       </c>
       <c r="E281" s="6" t="inlineStr">
         <is>
-          <t>_strategy_mode read but never written</t>
+          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
         </is>
       </c>
       <c r="F281" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
+          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
         </is>
       </c>
       <c r="G281" s="5" t="inlineStr">
         <is>
-          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
+          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr"/>
@@ -16208,23 +16208,23 @@
       </c>
       <c r="L281" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M281" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>93ec11842</t>
         </is>
       </c>
       <c r="N281" s="8" t="inlineStr"/>
     </row>
-    <row r="282" ht="105" customHeight="1">
+    <row r="282" ht="60" customHeight="1">
       <c r="A282" s="2" t="n">
         <v>281</v>
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>TRACKER-BUY-FILTER</t>
+          <t>TE-STRATEGY-MODE</t>
         </is>
       </c>
       <c r="C282" s="10" t="inlineStr">
@@ -16234,31 +16234,27 @@
       </c>
       <c r="D282" s="5" t="inlineStr">
         <is>
-          <t>Tracker/Feedback Loop</t>
+          <t>Target Engine</t>
         </is>
       </c>
       <c r="E282" s="6" t="inlineStr">
         <is>
-          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
+          <t>_strategy_mode read but never written</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
+          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
         </is>
       </c>
       <c r="G282" s="5" t="inlineStr">
         <is>
-          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr"/>
       <c r="I282" s="5" t="inlineStr"/>
-      <c r="J282" s="5" t="inlineStr">
-        <is>
-          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
-        </is>
-      </c>
+      <c r="J282" s="5" t="inlineStr"/>
       <c r="K282" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16266,27 +16262,23 @@
       </c>
       <c r="L282" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M282" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N282" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="283" ht="135" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N282" s="8" t="inlineStr"/>
+    </row>
+    <row r="283" ht="105" customHeight="1">
       <c r="A283" s="2" t="n">
         <v>282</v>
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
+          <t>TRACKER-BUY-FILTER</t>
         </is>
       </c>
       <c r="C283" s="10" t="inlineStr">
@@ -16296,37 +16288,29 @@
       </c>
       <c r="D283" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Tracker/Feedback Loop</t>
         </is>
       </c>
       <c r="E283" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
         </is>
       </c>
       <c r="G283" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
-        </is>
-      </c>
-      <c r="H283" s="2" t="inlineStr">
-        <is>
-          <t>1-2 hrs</t>
-        </is>
-      </c>
-      <c r="I283" s="5" t="inlineStr">
-        <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
-        </is>
-      </c>
+          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr"/>
+      <c r="I283" s="5" t="inlineStr"/>
       <c r="J283" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
         </is>
       </c>
       <c r="K283" s="12" t="inlineStr">
@@ -16336,27 +16320,27 @@
       </c>
       <c r="L283" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M283" s="3" t="inlineStr">
         <is>
-          <t>42c36ef91</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N283" s="8" t="inlineStr">
         <is>
-          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="284" ht="45" customHeight="1">
+          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="135" customHeight="1">
       <c r="A284" s="2" t="n">
         <v>283</v>
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>STOCKSMITH-BOOK-RISK</t>
+          <t>MOD-1</t>
         </is>
       </c>
       <c r="C284" s="10" t="inlineStr">
@@ -16366,27 +16350,39 @@
       </c>
       <c r="D284" s="5" t="inlineStr">
         <is>
-          <t>V2 Dashboard / Risk</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E284" s="6" t="inlineStr">
         <is>
-          <t>Book Risk surface + per-lens analytics (§6)</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G284" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
-        </is>
-      </c>
-      <c r="H284" s="2" t="inlineStr"/>
-      <c r="I284" s="5" t="inlineStr"/>
-      <c r="J284" s="5" t="inlineStr"/>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I284" s="5" t="inlineStr">
+        <is>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
+        </is>
+      </c>
+      <c r="J284" s="5" t="inlineStr">
+        <is>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+        </is>
+      </c>
       <c r="K284" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16394,23 +16390,27 @@
       </c>
       <c r="L284" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M284" s="3" t="inlineStr">
         <is>
-          <t>50cace567</t>
-        </is>
-      </c>
-      <c r="N284" s="8" t="inlineStr"/>
-    </row>
-    <row r="285" ht="120" customHeight="1">
+          <t>42c36ef91</t>
+        </is>
+      </c>
+      <c r="N284" s="8" t="inlineStr">
+        <is>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="45" customHeight="1">
       <c r="A285" s="2" t="n">
         <v>284</v>
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>RECENCY-FLOOR</t>
+          <t>STOCKSMITH-BOOK-RISK</t>
         </is>
       </c>
       <c r="C285" s="10" t="inlineStr">
@@ -16420,31 +16420,27 @@
       </c>
       <c r="D285" s="5" t="inlineStr">
         <is>
-          <t>Validation Hygiene</t>
+          <t>V2 Dashboard / Risk</t>
         </is>
       </c>
       <c r="E285" s="6" t="inlineStr">
         <is>
-          <t>_validations needs recency floor — auto-revert stale boosts</t>
+          <t>Book Risk surface + per-lens analytics (§6)</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
+          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
         </is>
       </c>
       <c r="G285" s="5" t="inlineStr">
         <is>
-          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
+          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr"/>
       <c r="I285" s="5" t="inlineStr"/>
-      <c r="J285" s="5" t="inlineStr">
-        <is>
-          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
-        </is>
-      </c>
+      <c r="J285" s="5" t="inlineStr"/>
       <c r="K285" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16452,27 +16448,23 @@
       </c>
       <c r="L285" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="M285" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N285" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="286" ht="60" customHeight="1">
+          <t>50cace567</t>
+        </is>
+      </c>
+      <c r="N285" s="8" t="inlineStr"/>
+    </row>
+    <row r="286" ht="120" customHeight="1">
       <c r="A286" s="2" t="n">
         <v>285</v>
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-TAB</t>
+          <t>RECENCY-FLOOR</t>
         </is>
       </c>
       <c r="C286" s="10" t="inlineStr">
@@ -16482,27 +16474,31 @@
       </c>
       <c r="D286" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Momentum</t>
+          <t>Validation Hygiene</t>
         </is>
       </c>
       <c r="E286" s="6" t="inlineStr">
         <is>
-          <t>New 🚀 Momentum workspace tab</t>
+          <t>_validations needs recency floor — auto-revert stale boosts</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
+          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
         </is>
       </c>
       <c r="G286" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
+          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr"/>
       <c r="I286" s="5" t="inlineStr"/>
-      <c r="J286" s="5" t="inlineStr"/>
+      <c r="J286" s="5" t="inlineStr">
+        <is>
+          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
+        </is>
+      </c>
       <c r="K286" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16510,15 +16506,19 @@
       </c>
       <c r="L286" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N286" s="8" t="inlineStr"/>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N286" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
+        </is>
+      </c>
     </row>
     <row r="287" ht="60" customHeight="1">
       <c r="A287" s="2" t="n">
@@ -16526,7 +16526,7 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-QUICK-PANELS</t>
+          <t>MOMENTUM-TAB</t>
         </is>
       </c>
       <c r="C287" s="10" t="inlineStr">
@@ -16536,22 +16536,22 @@
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Signal Scanner</t>
+          <t>Workspaces / Momentum</t>
         </is>
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>5 quick-glance panels above watchlist table</t>
+          <t>New 🚀 Momentum workspace tab</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
+          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
         </is>
       </c>
       <c r="G287" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr"/>
@@ -16569,60 +16569,48 @@
       </c>
       <c r="M287" s="3" t="inlineStr">
         <is>
-          <t>dfbe955fe</t>
+          <t>27fd646b1</t>
         </is>
       </c>
       <c r="N287" s="8" t="inlineStr"/>
     </row>
-    <row r="288" ht="45" customHeight="1">
+    <row r="288" ht="60" customHeight="1">
       <c r="A288" s="2" t="n">
         <v>287</v>
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C288" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>SCANNER-QUICK-PANELS</t>
+        </is>
+      </c>
+      <c r="C288" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D288" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Workspaces / Signal Scanner</t>
         </is>
       </c>
       <c r="E288" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>5 quick-glance panels above watchlist table</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
         </is>
       </c>
       <c r="G288" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
-        </is>
-      </c>
-      <c r="H288" s="2" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="I288" s="5" t="inlineStr">
-        <is>
-          <t>Win: persistence works; no silent overwrites.</t>
-        </is>
-      </c>
-      <c r="J288" s="5" t="inlineStr">
-        <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
-        </is>
-      </c>
+          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr"/>
+      <c r="I288" s="5" t="inlineStr"/>
+      <c r="J288" s="5" t="inlineStr"/>
       <c r="K288" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16630,15 +16618,15 @@
       </c>
       <c r="L288" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M288" s="3" t="inlineStr"/>
-      <c r="N288" s="8" t="inlineStr">
-        <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="M288" s="3" t="inlineStr">
+        <is>
+          <t>dfbe955fe</t>
+        </is>
+      </c>
+      <c r="N288" s="8" t="inlineStr"/>
     </row>
     <row r="289" ht="45" customHeight="1">
       <c r="A289" s="2" t="n">
@@ -16646,7 +16634,7 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="C289" s="13" t="inlineStr">
@@ -16661,32 +16649,32 @@
       </c>
       <c r="E289" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G289" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
-          <t>verified (no change needed)</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I289" s="5" t="inlineStr">
         <is>
-          <t>Win: confirms infrastructure still healthy.</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J289" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
         </is>
       </c>
       <c r="K289" s="12" t="inlineStr">
@@ -16702,7 +16690,7 @@
       <c r="M289" s="3" t="inlineStr"/>
       <c r="N289" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
         </is>
       </c>
     </row>
@@ -16712,7 +16700,7 @@
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>UI-3</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C290" s="13" t="inlineStr">
@@ -16722,35 +16710,39 @@
       </c>
       <c r="D290" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
         <is>
-          <t>Remove emoji icons from Thesis + Research labels</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
         <is>
-          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G290" s="5" t="inlineStr">
         <is>
-          <t>Removed emojis from FD sub-tab nav + section headers.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I290" s="5" t="inlineStr">
         <is>
-          <t>Low / cosmetic</t>
-        </is>
-      </c>
-      <c r="J290" s="5" t="inlineStr"/>
+          <t>Win: confirms infrastructure still healthy.</t>
+        </is>
+      </c>
+      <c r="J290" s="5" t="inlineStr">
+        <is>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
       <c r="K290" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16758,17 +16750,13 @@
       </c>
       <c r="L290" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="M290" s="3" t="inlineStr">
-        <is>
-          <t>24fd7c273</t>
-        </is>
-      </c>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M290" s="3" t="inlineStr"/>
       <c r="N290" s="8" t="inlineStr">
         <is>
-          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
         </is>
       </c>
     </row>
@@ -16778,59 +16766,63 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
-        </is>
-      </c>
-      <c r="C291" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>UI-3</t>
+        </is>
+      </c>
+      <c r="C291" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D291" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E291" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Remove emoji icons from Thesis + Research labels</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
         </is>
       </c>
       <c r="G291" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+          <t>Removed emojis from FD sub-tab nav + section headers.</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>5 min after answer</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I291" s="5" t="inlineStr">
         <is>
-          <t>Win: -671 lines.</t>
-        </is>
-      </c>
-      <c r="J291" s="5" t="inlineStr">
-        <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K291" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L291" s="2" t="inlineStr"/>
-      <c r="M291" s="3" t="inlineStr"/>
+          <t>Low / cosmetic</t>
+        </is>
+      </c>
+      <c r="J291" s="5" t="inlineStr"/>
+      <c r="K291" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L291" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M291" s="3" t="inlineStr">
+        <is>
+          <t>24fd7c273</t>
+        </is>
+      </c>
       <c r="N291" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
         </is>
       </c>
     </row>
@@ -16840,7 +16832,7 @@
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
+          <t>CLEAN-2</t>
         </is>
       </c>
       <c r="C292" s="10" t="inlineStr">
@@ -16850,37 +16842,37 @@
       </c>
       <c r="D292" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E292" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
         </is>
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
         </is>
       </c>
       <c r="G292" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>5 min after answer</t>
         </is>
       </c>
       <c r="I292" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Win: -671 lines.</t>
         </is>
       </c>
       <c r="J292" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
+          <t>Standard data-migration retention practice.</t>
         </is>
       </c>
       <c r="K292" s="14" t="inlineStr">
@@ -16902,109 +16894,109 @@
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C293" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C293" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D293" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E293" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
         </is>
       </c>
       <c r="G293" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
         </is>
       </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>hours-days each</t>
         </is>
       </c>
       <c r="I293" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win varies; defer until PERF-7 measured.</t>
         </is>
       </c>
       <c r="J293" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K293" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K293" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="L293" s="2" t="inlineStr"/>
       <c r="M293" s="3" t="inlineStr"/>
       <c r="N293" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="294" ht="75" customHeight="1">
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="45" customHeight="1">
       <c r="A294" s="2" t="n">
         <v>293</v>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>MOD-2</t>
-        </is>
-      </c>
-      <c r="C294" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C294" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D294" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E294" s="6" t="inlineStr">
         <is>
-          <t>Pixel-diff regression baseline</t>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
         </is>
       </c>
       <c r="F294" s="5" t="inlineStr">
         <is>
-          <t>After modularization, no automated visual-regression catch.</t>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
         </is>
       </c>
       <c r="G294" s="5" t="inlineStr">
         <is>
-          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I294" s="5" t="inlineStr">
         <is>
-          <t>Win: catches accidental layout regressions.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J294" s="5" t="inlineStr">
         <is>
-          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+          <t>Agents skim and miss post-filter subset analysis.</t>
         </is>
       </c>
       <c r="K294" s="15" t="inlineStr">
@@ -17012,147 +17004,209 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L294" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
+      <c r="L294" s="2" t="inlineStr"/>
       <c r="M294" s="3" t="inlineStr"/>
       <c r="N294" s="8" t="inlineStr">
         <is>
-          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="295" ht="195" customHeight="1">
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="75" customHeight="1">
       <c r="A295" s="2" t="n">
         <v>294</v>
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
+          <t>MOD-2</t>
+        </is>
+      </c>
+      <c r="C295" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D295" s="5" t="inlineStr">
+        <is>
+          <t>UI / Modularization</t>
+        </is>
+      </c>
+      <c r="E295" s="6" t="inlineStr">
+        <is>
+          <t>Pixel-diff regression baseline</t>
+        </is>
+      </c>
+      <c r="F295" s="5" t="inlineStr">
+        <is>
+          <t>After modularization, no automated visual-regression catch.</t>
+        </is>
+      </c>
+      <c r="G295" s="5" t="inlineStr">
+        <is>
+          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+        </is>
+      </c>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t>2-3 hrs</t>
+        </is>
+      </c>
+      <c r="I295" s="5" t="inlineStr">
+        <is>
+          <t>Win: catches accidental layout regressions.</t>
+        </is>
+      </c>
+      <c r="J295" s="5" t="inlineStr">
+        <is>
+          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+        </is>
+      </c>
+      <c r="K295" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L295" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="M295" s="3" t="inlineStr"/>
+      <c r="N295" s="8" t="inlineStr">
+        <is>
+          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="195" customHeight="1">
+      <c r="A296" s="2" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
           <t>OB-CONFLUENCE-PROPOSAL-REJECTED</t>
         </is>
       </c>
-      <c r="C295" s="10" t="inlineStr">
+      <c r="C296" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D295" s="5" t="inlineStr">
+      <c r="D296" s="5" t="inlineStr">
         <is>
           <t>Signals / Cross-Check</t>
         </is>
       </c>
-      <c r="E295" s="6" t="inlineStr">
+      <c r="E296" s="6" t="inlineStr">
         <is>
           <t>OB-confluence Wilson bump + OB-aware stop — proposals KILLED by backtest evidence</t>
         </is>
       </c>
-      <c r="F295" s="5" t="inlineStr">
+      <c r="F296" s="5" t="inlineStr">
         <is>
           <t>User asked 2026-05-12 to ship #2 (Wilson-bump score factor for bullish OB confluence within 5% of entry) and #5 (OB-low as stop instead of 1.25xATR). Per Principle 1 / Principle 7, ran post-hoc validation: scripts/validate_ob_confluence.py retroactively tags every closed trade from existing portfolio_backtest outputs with SMC state at entry date, computes Wilson 95% LB per subset.
 RESULT (750-day backtest · n=384): Bull OB confluence within 5% of entry DECREASES Wilson LB by -8.6pp (14.6% vs baseline 23.1%). BOS-bullish boost: -3.4pp. SMC-bullish direction boost: -3.6pp. Per #5 simulation, 35 of 39 (90%) OB-low-as-stop would have loosened the stop; 25 of those still ended in losses (looser stops do not rescue broken setups, they extend exposure).
 Principle 4 fires: proposals FALSIFIED, killed permanently (not retuned). Doing the change without this validation would have introduced a 6-9pp Wilson-LB drag on every BUY signal.</t>
         </is>
       </c>
-      <c r="G295" s="5" t="inlineStr">
+      <c r="G296" s="5" t="inlineStr">
         <is>
           <t>Built scripts/validate_ob_confluence.py to retroactively run smart_money.score_smc() on the historical OHLCV at each trade's entry date, tag with OB-confluence + BOS + CHoCH flags, compute Wilson 95% LB per subset, and apply Principle 1 gates (n&gt;=30, lift&gt;=5pp). Cross-validated on 250d (n=142) and 750d (n=384) backtest outputs. Both agree: NO EDGE.</t>
         </is>
       </c>
-      <c r="H295" s="2" t="inlineStr">
+      <c r="H296" s="2" t="inlineStr">
         <is>
           <t>Days of work avoided (would have shipped a degrading change).</t>
         </is>
       </c>
-      <c r="I295" s="5" t="inlineStr">
+      <c r="I296" s="5" t="inlineStr">
         <is>
           <t>Mechanism (Principle 2): institutional OBs are supposed to mark re-add zones for smart money. Falsification (Principle 4): if the data doesn't show OB-confluent trades winning more, the mechanism either doesn't exist for retail-accessible OB detection at daily resolution OR is already priced into our 5-pillar score. Either way: ship nothing. The proposals are dead. Win: prevented a 6-9pp Wilson-LB drag from being added to live scoring. Lost: nothing — we didn't change live scoring, no opportunity cost.</t>
         </is>
       </c>
-      <c r="J295" s="5" t="inlineStr">
+      <c r="J296" s="5" t="inlineStr">
         <is>
           <t>Validator script is reusable infrastructure. Re-run any time the SMC detection logic or score thresholds change. NOTE: baseline WR in 750d backtest is 27.3% (low) — the absolute level reflects backtest-window-specific market conditions; the SUBSET comparisons are valid regardless because they share the same baseline. Do not interpret 23.1% Wilson LB as a system-level edge — that's a separate question. This validation answers ONLY: does OB-confluence improve selection within whatever the system already does.</t>
         </is>
       </c>
-      <c r="K295" s="15" t="inlineStr">
+      <c r="K296" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L295" s="2" t="inlineStr">
+      <c r="L296" s="2" t="inlineStr">
         <is>
           <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="M295" s="3" t="inlineStr"/>
-      <c r="N295" s="8" t="inlineStr">
-        <is>
-          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="296" ht="90" customHeight="1">
-      <c r="A296" s="2" t="n">
-        <v>295</v>
-      </c>
-      <c r="B296" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C296" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="D296" s="5" t="inlineStr">
-        <is>
-          <t>Data / Universe</t>
-        </is>
-      </c>
-      <c r="E296" s="6" t="inlineStr">
-        <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
-        </is>
-      </c>
-      <c r="F296" s="5" t="inlineStr">
-        <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
-        </is>
-      </c>
-      <c r="G296" s="5" t="inlineStr">
-        <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
-        </is>
-      </c>
-      <c r="H296" s="2" t="inlineStr">
-        <is>
-          <t>$$ + 1 day</t>
-        </is>
-      </c>
-      <c r="I296" s="5" t="inlineStr">
-        <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
-        </is>
-      </c>
-      <c r="J296" s="5" t="inlineStr">
-        <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K296" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L296" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr"/>
       <c r="N296" s="8" t="inlineStr">
+        <is>
+          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="90" customHeight="1">
+      <c r="A297" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C297" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D297" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E297" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F297" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G297" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H297" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I297" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J297" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K297" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L297" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M297" s="3" t="inlineStr"/>
+      <c r="N297" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -17257,10 +17311,10 @@
         <v>86</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5">
@@ -17314,10 +17368,10 @@
         <v>111</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>